<commit_message>
LVBR-605 Bewindvoerder als nieuw contacttype
</commit_message>
<xml_diff>
--- a/src/main/resources/be/vlaanderen/omgeving/data/id/conceptscheme/verwaarlozing/verwaarlozing.xlsx
+++ b/src/main/resources/be/vlaanderen/omgeving/data/id/conceptscheme/verwaarlozing/verwaarlozing.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S70"/>
+  <dimension ref="A1:S71"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1758,7 +1758,7 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/rol/curator</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/rol/bewindvoerder</v>
       </c>
       <c r="B24" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -1773,7 +1773,7 @@
         <v>null</v>
       </c>
       <c r="F24" t="str">
-        <v>Curator</v>
+        <v>Bewindvoerder</v>
       </c>
       <c r="G24" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/rol</v>
@@ -1817,7 +1817,7 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/rol/eigenaar</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/rol/curator</v>
       </c>
       <c r="B25" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -1832,16 +1832,16 @@
         <v>null</v>
       </c>
       <c r="F25" t="str">
-        <v>Eigenaar</v>
+        <v>Curator</v>
       </c>
       <c r="G25" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/rol</v>
       </c>
       <c r="H25" t="str">
-        <v>De houder van een van de volgende zakelijke rechten met betrekking tot een bedrijfsgebouw: de volle eigendom, het recht van opstal of van erfpacht, het vruchtgebruik</v>
+        <v>null</v>
       </c>
       <c r="I25" t="str">
-        <v>De houder van een van de volgende zakelijke rechten met betrekking tot een bedrijfsgebouw: de volle eigendom, het recht van opstal of van erfpacht, het vruchtgebruik</v>
+        <v>null</v>
       </c>
       <c r="J25" t="str">
         <v>null</v>
@@ -1876,7 +1876,7 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/rol/instrumenterend_ambtenaar</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/rol/eigenaar</v>
       </c>
       <c r="B26" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -1891,16 +1891,16 @@
         <v>null</v>
       </c>
       <c r="F26" t="str">
-        <v>Instrumenterend ambtenaar</v>
+        <v>Eigenaar</v>
       </c>
       <c r="G26" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/rol</v>
       </c>
       <c r="H26" t="str">
-        <v>Iedere persoon of instelling die ertoe gemachtigd is aktes van eigendomsoverdracht te verlijden</v>
+        <v>De houder van een van de volgende zakelijke rechten met betrekking tot een bedrijfsgebouw: de volle eigendom, het recht van opstal of van erfpacht, het vruchtgebruik</v>
       </c>
       <c r="I26" t="str">
-        <v>Iedere persoon of instelling die ertoe gemachtigd is aktes van eigendomsoverdracht te verlijden</v>
+        <v>De houder van een van de volgende zakelijke rechten met betrekking tot een bedrijfsgebouw: de volle eigendom, het recht van opstal of van erfpacht, het vruchtgebruik</v>
       </c>
       <c r="J26" t="str">
         <v>null</v>
@@ -1935,7 +1935,7 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/rol/raadsman</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/rol/instrumenterend_ambtenaar</v>
       </c>
       <c r="B27" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -1950,16 +1950,16 @@
         <v>null</v>
       </c>
       <c r="F27" t="str">
-        <v>Raadsman</v>
+        <v>Instrumenterend ambtenaar</v>
       </c>
       <c r="G27" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/rol</v>
       </c>
       <c r="H27" t="str">
-        <v>null</v>
+        <v>Iedere persoon of instelling die ertoe gemachtigd is aktes van eigendomsoverdracht te verlijden</v>
       </c>
       <c r="I27" t="str">
-        <v>null</v>
+        <v>Iedere persoon of instelling die ertoe gemachtigd is aktes van eigendomsoverdracht te verlijden</v>
       </c>
       <c r="J27" t="str">
         <v>null</v>
@@ -1994,25 +1994,25 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_aanvaard</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/rol/raadsman</v>
       </c>
       <c r="B28" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C28" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/aanvraag_opschorting_heffing_aanvaard</v>
+        <v>null</v>
       </c>
       <c r="D28" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/rol</v>
       </c>
       <c r="E28" t="str">
-        <v>OPSCH_ANVRD</v>
+        <v>null</v>
       </c>
       <c r="F28" t="str">
-        <v>Opschorting aanvaard</v>
+        <v>Raadsman</v>
       </c>
       <c r="G28" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/rol</v>
       </c>
       <c r="H28" t="str">
         <v>null</v>
@@ -2021,13 +2021,13 @@
         <v>null</v>
       </c>
       <c r="J28" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
+        <v>null</v>
       </c>
       <c r="K28" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
+        <v>null</v>
       </c>
       <c r="L28" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
+        <v>null</v>
       </c>
       <c r="M28" t="str">
         <v>null</v>
@@ -2053,22 +2053,22 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_aanvaard_begeleidende_brief</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_aanvaard</v>
       </c>
       <c r="B29" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C29" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_aanvaard</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/aanvraag_opschorting_heffing_aanvaard</v>
       </c>
       <c r="D29" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E29" t="str">
-        <v>OPSCH_ANVRD_BEG_BRIEF</v>
+        <v>OPSCH_ANVRD</v>
       </c>
       <c r="F29" t="str">
-        <v>Begeleidende brief bij opschorting aanvaard</v>
+        <v>Opschorting aanvaard</v>
       </c>
       <c r="G29" t="str">
         <v>null</v>
@@ -2112,22 +2112,22 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_niet_aanvaard</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_aanvaard_begeleidende_brief</v>
       </c>
       <c r="B30" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C30" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/aanvraag_opschorting_heffing_niet_aanvaard</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_aanvaard</v>
       </c>
       <c r="D30" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E30" t="str">
-        <v>OPSCH_NANVRD</v>
+        <v>OPSCH_ANVRD_BEG_BRIEF</v>
       </c>
       <c r="F30" t="str">
-        <v>Opschorting niet aanvaard</v>
+        <v>Begeleidende brief bij opschorting aanvaard</v>
       </c>
       <c r="G30" t="str">
         <v>null</v>
@@ -2171,22 +2171,22 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_niet_aanvaard_begeleidende_brief</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_niet_aanvaard</v>
       </c>
       <c r="B31" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C31" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_niet_aanvaard</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/aanvraag_opschorting_heffing_niet_aanvaard</v>
       </c>
       <c r="D31" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E31" t="str">
-        <v>OPSCH_NANVRD_BEG_BRIEF</v>
+        <v>OPSCH_NANVRD</v>
       </c>
       <c r="F31" t="str">
-        <v>Begeleidende brief bij opschorting niet aanvaard</v>
+        <v>Opschorting niet aanvaard</v>
       </c>
       <c r="G31" t="str">
         <v>null</v>
@@ -2230,22 +2230,22 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_aanvaard</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_niet_aanvaard_begeleidende_brief</v>
       </c>
       <c r="B32" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C32" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/aanvraag_schrapping_aanvaard</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_niet_aanvaard</v>
       </c>
       <c r="D32" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E32" t="str">
-        <v>SCHR_ANVRD</v>
+        <v>OPSCH_NANVRD_BEG_BRIEF</v>
       </c>
       <c r="F32" t="str">
-        <v>Schrapping aanvaard</v>
+        <v>Begeleidende brief bij opschorting niet aanvaard</v>
       </c>
       <c r="G32" t="str">
         <v>null</v>
@@ -2289,22 +2289,22 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_aanvaard_begeleidende_brief</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_aanvaard</v>
       </c>
       <c r="B33" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C33" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_aanvaard</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/aanvraag_schrapping_aanvaard</v>
       </c>
       <c r="D33" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E33" t="str">
-        <v>SCHR_ANVRD_BEG_BRIEF</v>
+        <v>SCHR_ANVRD</v>
       </c>
       <c r="F33" t="str">
-        <v>Begeleidende brief bij schrapping aanvaard</v>
+        <v>Schrapping aanvaard</v>
       </c>
       <c r="G33" t="str">
         <v>null</v>
@@ -2348,22 +2348,22 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_niet_aanvaard</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_aanvaard_begeleidende_brief</v>
       </c>
       <c r="B34" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C34" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/aanvraag_schrapping_niet_aanvaard</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_aanvaard</v>
       </c>
       <c r="D34" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E34" t="str">
-        <v>SCHR_NANVRD</v>
+        <v>SCHR_ANVRD_BEG_BRIEF</v>
       </c>
       <c r="F34" t="str">
-        <v>Schrapping niet aanvaard</v>
+        <v>Begeleidende brief bij schrapping aanvaard</v>
       </c>
       <c r="G34" t="str">
         <v>null</v>
@@ -2407,22 +2407,22 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_niet_aanvaard_begeleidende_brief</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_niet_aanvaard</v>
       </c>
       <c r="B35" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C35" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_niet_aanvaard</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/aanvraag_schrapping_niet_aanvaard</v>
       </c>
       <c r="D35" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E35" t="str">
-        <v>SCHR_NANVRD_BEG_BRIEF</v>
+        <v>SCHR_NANVRD</v>
       </c>
       <c r="F35" t="str">
-        <v>Begeleidende brief bij schrapping niet aanvaard</v>
+        <v>Schrapping niet aanvaard</v>
       </c>
       <c r="G35" t="str">
         <v>null</v>
@@ -2466,22 +2466,22 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_ingewilligd</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_niet_aanvaard_begeleidende_brief</v>
       </c>
       <c r="B36" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C36" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/beroep_tegen_registratie_ingewilligd</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_niet_aanvaard</v>
       </c>
       <c r="D36" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E36" t="str">
-        <v>BER_INGWD</v>
+        <v>SCHR_NANVRD_BEG_BRIEF</v>
       </c>
       <c r="F36" t="str">
-        <v>Beroep ingewilligd</v>
+        <v>Begeleidende brief bij schrapping niet aanvaard</v>
       </c>
       <c r="G36" t="str">
         <v>null</v>
@@ -2525,22 +2525,22 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_ingewilligd_begeleidende_brief</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_ingewilligd</v>
       </c>
       <c r="B37" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C37" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_ingewilligd</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/beroep_tegen_registratie_ingewilligd</v>
       </c>
       <c r="D37" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E37" t="str">
-        <v>BER_INGWD_BEG_BRIEF</v>
+        <v>BER_INGWD</v>
       </c>
       <c r="F37" t="str">
-        <v>Begeleidende brief bij beroep ingewilligd</v>
+        <v>Beroep ingewilligd</v>
       </c>
       <c r="G37" t="str">
         <v>null</v>
@@ -2584,22 +2584,22 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_onontvankelijk_verklaard</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_ingewilligd_begeleidende_brief</v>
       </c>
       <c r="B38" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C38" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/beroep_tegen_registratie_onontvankelijk_verklaard</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_ingewilligd</v>
       </c>
       <c r="D38" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E38" t="str">
-        <v>BER_ON</v>
+        <v>BER_INGWD_BEG_BRIEF</v>
       </c>
       <c r="F38" t="str">
-        <v>Beroep onontvankelijk verklaard</v>
+        <v>Begeleidende brief bij beroep ingewilligd</v>
       </c>
       <c r="G38" t="str">
         <v>null</v>
@@ -2643,22 +2643,22 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_onontvankelijk_verklaard_begeleidende_brief</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_onontvankelijk_verklaard</v>
       </c>
       <c r="B39" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C39" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_onontvankelijk_verklaard</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/beroep_tegen_registratie_onontvankelijk_verklaard</v>
       </c>
       <c r="D39" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E39" t="str">
-        <v>BER_ON_BEG_BRIEF</v>
+        <v>BER_ON</v>
       </c>
       <c r="F39" t="str">
-        <v>Begeleidende brief bij beroep onontvankelijk verklaard</v>
+        <v>Beroep onontvankelijk verklaard</v>
       </c>
       <c r="G39" t="str">
         <v>null</v>
@@ -2702,22 +2702,22 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_verworpen</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_onontvankelijk_verklaard_begeleidende_brief</v>
       </c>
       <c r="B40" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C40" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/beroep_tegen_registratie_verworpen</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_onontvankelijk_verklaard</v>
       </c>
       <c r="D40" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E40" t="str">
-        <v>BER_VERWN</v>
+        <v>BER_ON_BEG_BRIEF</v>
       </c>
       <c r="F40" t="str">
-        <v>Beroep verworpen</v>
+        <v>Begeleidende brief bij beroep onontvankelijk verklaard</v>
       </c>
       <c r="G40" t="str">
         <v>null</v>
@@ -2761,22 +2761,22 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_verworpen_begeleidende_brief</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_verworpen</v>
       </c>
       <c r="B41" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C41" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_verworpen</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/beroep_tegen_registratie_verworpen</v>
       </c>
       <c r="D41" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E41" t="str">
-        <v>BER_VERWN_BEG_BRIEF</v>
+        <v>BER_VERWN</v>
       </c>
       <c r="F41" t="str">
-        <v>Begeleidende brief bij beroep verworpen</v>
+        <v>Beroep verworpen</v>
       </c>
       <c r="G41" t="str">
         <v>null</v>
@@ -2820,25 +2820,25 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_verworpen_begeleidende_brief</v>
       </c>
       <c r="B42" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C42" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_verworpen</v>
       </c>
       <c r="D42" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E42" t="str">
-        <v>beslissingsstuk</v>
+        <v>BER_VERWN_BEG_BRIEF</v>
       </c>
       <c r="F42" t="str">
-        <v>Stuk dat voortkomt uit een beslissing</v>
+        <v>Begeleidende brief bij beroep verworpen</v>
       </c>
       <c r="G42" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
+        <v>null</v>
       </c>
       <c r="H42" t="str">
         <v>null</v>
@@ -2847,19 +2847,19 @@
         <v>null</v>
       </c>
       <c r="J42" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
       </c>
       <c r="K42" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
       </c>
       <c r="L42" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_niet_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_niet_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_niet_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_niet_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_ingewilligd|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_ingewilligd_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_onontvankelijk_verklaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_onontvankelijk_verklaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_verworpen|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_verworpen_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/registratieattest|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/registratieattest_begeleidende_brief</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
       </c>
       <c r="M42" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_niet_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_niet_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_niet_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_niet_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_ingewilligd|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_ingewilligd_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_onontvankelijk_verklaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_onontvankelijk_verklaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_verworpen|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_verworpen_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/registratieattest|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/registratieattest_begeleidende_brief</v>
+        <v>null</v>
       </c>
       <c r="N42" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_niet_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_niet_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_niet_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_niet_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_ingewilligd|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_ingewilligd_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_onontvankelijk_verklaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_onontvankelijk_verklaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_verworpen|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_verworpen_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/registratieattest|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/registratieattest_begeleidende_brief</v>
+        <v>null</v>
       </c>
       <c r="O42" t="str">
         <v>null</v>
@@ -2879,7 +2879,7 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/foto</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
       </c>
       <c r="B43" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -2891,13 +2891,13 @@
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E43" t="str">
-        <v>FOTO</v>
+        <v>beslissingsstuk</v>
       </c>
       <c r="F43" t="str">
-        <v>Foto</v>
+        <v>Stuk dat voortkomt uit een beslissing</v>
       </c>
       <c r="G43" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="H43" t="str">
         <v>null</v>
@@ -2906,19 +2906,19 @@
         <v>null</v>
       </c>
       <c r="J43" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/stavingsstuk</v>
+        <v>null</v>
       </c>
       <c r="K43" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/stavingsstuk</v>
+        <v>null</v>
       </c>
       <c r="L43" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/stavingsstuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_niet_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_niet_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_niet_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_niet_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_ingewilligd|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_ingewilligd_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_onontvankelijk_verklaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_onontvankelijk_verklaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_verworpen|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_verworpen_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/registratieattest|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/registratieattest_begeleidende_brief</v>
       </c>
       <c r="M43" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_niet_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_niet_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_niet_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_niet_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_ingewilligd|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_ingewilligd_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_onontvankelijk_verklaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_onontvankelijk_verklaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_verworpen|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_verworpen_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/registratieattest|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/registratieattest_begeleidende_brief</v>
       </c>
       <c r="N43" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_niet_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_niet_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_niet_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_niet_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_ingewilligd|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_ingewilligd_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_onontvankelijk_verklaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_onontvankelijk_verklaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_verworpen|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_verworpen_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/registratieattest|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/registratieattest_begeleidende_brief</v>
       </c>
       <c r="O43" t="str">
         <v>null</v>
@@ -2938,7 +2938,7 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/inkomend_procedurestuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/foto</v>
       </c>
       <c r="B44" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -2950,10 +2950,10 @@
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E44" t="str">
-        <v>INKOMEND_PROCEDURESTUK</v>
+        <v>FOTO</v>
       </c>
       <c r="F44" t="str">
-        <v>Inkomend procedurestuk</v>
+        <v>Foto</v>
       </c>
       <c r="G44" t="str">
         <v>null</v>
@@ -2965,13 +2965,13 @@
         <v>null</v>
       </c>
       <c r="J44" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/procedurestuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/stavingsstuk</v>
       </c>
       <c r="K44" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/procedurestuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/stavingsstuk</v>
       </c>
       <c r="L44" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/procedurestuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/stavingsstuk</v>
       </c>
       <c r="M44" t="str">
         <v>null</v>
@@ -2997,7 +2997,7 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/procedurestuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/inkomend_procedurestuk</v>
       </c>
       <c r="B45" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -3009,13 +3009,13 @@
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E45" t="str">
-        <v>procedurestuk</v>
+        <v>INKOMEND_PROCEDURESTUK</v>
       </c>
       <c r="F45" t="str">
-        <v>Stuk gerelateerd aan een procedure</v>
+        <v>Inkomend procedurestuk</v>
       </c>
       <c r="G45" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
+        <v>null</v>
       </c>
       <c r="H45" t="str">
         <v>null</v>
@@ -3024,19 +3024,19 @@
         <v>null</v>
       </c>
       <c r="J45" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/procedurestuk</v>
       </c>
       <c r="K45" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/procedurestuk</v>
       </c>
       <c r="L45" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/inkomend_procedurestuk|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/retour_afzender_procedurestuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/procedurestuk</v>
       </c>
       <c r="M45" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/inkomend_procedurestuk|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/retour_afzender_procedurestuk</v>
+        <v>null</v>
       </c>
       <c r="N45" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/inkomend_procedurestuk|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/retour_afzender_procedurestuk</v>
+        <v>null</v>
       </c>
       <c r="O45" t="str">
         <v>null</v>
@@ -3056,25 +3056,25 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/registratieattest</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/procedurestuk</v>
       </c>
       <c r="B46" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C46" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/geregistreerd_in_inventaris</v>
+        <v>null</v>
       </c>
       <c r="D46" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E46" t="str">
-        <v>REGATT</v>
+        <v>procedurestuk</v>
       </c>
       <c r="F46" t="str">
-        <v>Registratieattest</v>
+        <v>Stuk gerelateerd aan een procedure</v>
       </c>
       <c r="G46" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="H46" t="str">
         <v>null</v>
@@ -3083,19 +3083,19 @@
         <v>null</v>
       </c>
       <c r="J46" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
+        <v>null</v>
       </c>
       <c r="K46" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
+        <v>null</v>
       </c>
       <c r="L46" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/inkomend_procedurestuk|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/retour_afzender_procedurestuk</v>
       </c>
       <c r="M46" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/inkomend_procedurestuk|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/retour_afzender_procedurestuk</v>
       </c>
       <c r="N46" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/inkomend_procedurestuk|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/retour_afzender_procedurestuk</v>
       </c>
       <c r="O46" t="str">
         <v>null</v>
@@ -3115,22 +3115,22 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/registratieattest_begeleidende_brief</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/registratieattest</v>
       </c>
       <c r="B47" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C47" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/geregistreerd_in_inventaris</v>
       </c>
       <c r="D47" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E47" t="str">
-        <v>REGATT_BEG_BRIEF</v>
+        <v>REGATT</v>
       </c>
       <c r="F47" t="str">
-        <v>Begeleidende brief bij een registratieattest</v>
+        <v>Registratieattest</v>
       </c>
       <c r="G47" t="str">
         <v>null</v>
@@ -3174,7 +3174,7 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/retour_afzender_procedurestuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/registratieattest_begeleidende_brief</v>
       </c>
       <c r="B48" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -3186,10 +3186,10 @@
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E48" t="str">
-        <v>RETOUR_AFZENDER_PROCEDURESTUK</v>
+        <v>REGATT_BEG_BRIEF</v>
       </c>
       <c r="F48" t="str">
-        <v>Retour afzender</v>
+        <v>Begeleidende brief bij een registratieattest</v>
       </c>
       <c r="G48" t="str">
         <v>null</v>
@@ -3201,13 +3201,13 @@
         <v>null</v>
       </c>
       <c r="J48" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/procedurestuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
       </c>
       <c r="K48" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/procedurestuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
       </c>
       <c r="L48" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/procedurestuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
       </c>
       <c r="M48" t="str">
         <v>null</v>
@@ -3233,7 +3233,7 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/stavingsstuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/retour_afzender_procedurestuk</v>
       </c>
       <c r="B49" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -3245,13 +3245,13 @@
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E49" t="str">
-        <v>stavingsstuk</v>
+        <v>RETOUR_AFZENDER_PROCEDURESTUK</v>
       </c>
       <c r="F49" t="str">
-        <v>Stavingsstuk bij een vaststelling</v>
+        <v>Retour afzender</v>
       </c>
       <c r="G49" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
+        <v>null</v>
       </c>
       <c r="H49" t="str">
         <v>null</v>
@@ -3260,19 +3260,19 @@
         <v>null</v>
       </c>
       <c r="J49" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/procedurestuk</v>
       </c>
       <c r="K49" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/procedurestuk</v>
       </c>
       <c r="L49" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/foto|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/varia|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/verslag</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/procedurestuk</v>
       </c>
       <c r="M49" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/foto|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/varia|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/verslag</v>
+        <v>null</v>
       </c>
       <c r="N49" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/foto|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/varia|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/verslag</v>
+        <v>null</v>
       </c>
       <c r="O49" t="str">
         <v>null</v>
@@ -3292,7 +3292,7 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/varia</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/stavingsstuk</v>
       </c>
       <c r="B50" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -3304,13 +3304,13 @@
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E50" t="str">
-        <v>VARIA</v>
+        <v>stavingsstuk</v>
       </c>
       <c r="F50" t="str">
-        <v>Varia</v>
+        <v>Stavingsstuk bij een vaststelling</v>
       </c>
       <c r="G50" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="H50" t="str">
         <v>null</v>
@@ -3319,19 +3319,19 @@
         <v>null</v>
       </c>
       <c r="J50" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/stavingsstuk</v>
+        <v>null</v>
       </c>
       <c r="K50" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/stavingsstuk</v>
+        <v>null</v>
       </c>
       <c r="L50" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/stavingsstuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/foto|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/varia|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/verslag</v>
       </c>
       <c r="M50" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/foto|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/varia|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/verslag</v>
       </c>
       <c r="N50" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/foto|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/varia|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/verslag</v>
       </c>
       <c r="O50" t="str">
         <v>null</v>
@@ -3351,7 +3351,7 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/verslag</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/varia</v>
       </c>
       <c r="B51" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -3363,10 +3363,10 @@
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E51" t="str">
-        <v>VERSLAG</v>
+        <v>VARIA</v>
       </c>
       <c r="F51" t="str">
-        <v>Verslag</v>
+        <v>Varia</v>
       </c>
       <c r="G51" t="str">
         <v>null</v>
@@ -3410,7 +3410,7 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/buitenmuren</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/verslag</v>
       </c>
       <c r="B52" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -3419,13 +3419,13 @@
         <v>null</v>
       </c>
       <c r="D52" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/uitgesproken_gebrek</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E52" t="str">
-        <v>buitenmuren</v>
+        <v>VERSLAG</v>
       </c>
       <c r="F52" t="str">
-        <v>Gebrek aan de toestand van buitenmuren</v>
+        <v>Verslag</v>
       </c>
       <c r="G52" t="str">
         <v>null</v>
@@ -3437,13 +3437,13 @@
         <v>null</v>
       </c>
       <c r="J52" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/stavingsstuk</v>
       </c>
       <c r="K52" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/stavingsstuk</v>
       </c>
       <c r="L52" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/stavingsstuk</v>
       </c>
       <c r="M52" t="str">
         <v>null</v>
@@ -3452,13 +3452,13 @@
         <v>null</v>
       </c>
       <c r="O52" t="str">
-        <v>Buitenmuren</v>
+        <v>null</v>
       </c>
       <c r="P52" t="str">
-        <v>http://www.eionet.europa.eu/gemet/theme/5</v>
+        <v>null</v>
       </c>
       <c r="Q52" t="str">
-        <v>https://data.omgeving.vlaanderen.be/ns/verwaarlozing#vertoont_gebrek_ivm_buitenmuren</v>
+        <v>null</v>
       </c>
       <c r="R52" t="str">
         <v>null</v>
@@ -3469,7 +3469,7 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/buitentimmerwerk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/buitenmuren</v>
       </c>
       <c r="B53" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -3481,10 +3481,10 @@
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/uitgesproken_gebrek</v>
       </c>
       <c r="E53" t="str">
-        <v>buitentimmerwerk</v>
+        <v>buitenmuren</v>
       </c>
       <c r="F53" t="str">
-        <v>Gebrek aan de toestand van het buitentimmerwerk</v>
+        <v>Gebrek aan de toestand van buitenmuren</v>
       </c>
       <c r="G53" t="str">
         <v>null</v>
@@ -3511,13 +3511,13 @@
         <v>null</v>
       </c>
       <c r="O53" t="str">
-        <v>Buitentimmerwerk</v>
+        <v>Buitenmuren</v>
       </c>
       <c r="P53" t="str">
         <v>http://www.eionet.europa.eu/gemet/theme/5</v>
       </c>
       <c r="Q53" t="str">
-        <v>https://data.omgeving.vlaanderen.be/ns/verwaarlozing#vertoont_gebrek_ivm_buitentimmerwerk</v>
+        <v>https://data.omgeving.vlaanderen.be/ns/verwaarlozing#vertoont_gebrek_ivm_buitenmuren</v>
       </c>
       <c r="R53" t="str">
         <v>null</v>
@@ -3528,7 +3528,7 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakbedekking</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/buitentimmerwerk</v>
       </c>
       <c r="B54" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -3540,10 +3540,10 @@
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/uitgesproken_gebrek</v>
       </c>
       <c r="E54" t="str">
-        <v>dakbedekking</v>
+        <v>buitentimmerwerk</v>
       </c>
       <c r="F54" t="str">
-        <v>Gebrek aan de toestand van de dakbedekking</v>
+        <v>Gebrek aan de toestand van het buitentimmerwerk</v>
       </c>
       <c r="G54" t="str">
         <v>null</v>
@@ -3570,13 +3570,13 @@
         <v>null</v>
       </c>
       <c r="O54" t="str">
-        <v>Dakbedekking</v>
+        <v>Buitentimmerwerk</v>
       </c>
       <c r="P54" t="str">
         <v>http://www.eionet.europa.eu/gemet/theme/5</v>
       </c>
       <c r="Q54" t="str">
-        <v>https://data.omgeving.vlaanderen.be/ns/verwaarlozing#vertoont_gebrek_ivm_dakbedekking</v>
+        <v>https://data.omgeving.vlaanderen.be/ns/verwaarlozing#vertoont_gebrek_ivm_buitentimmerwerk</v>
       </c>
       <c r="R54" t="str">
         <v>null</v>
@@ -3587,7 +3587,7 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakgebinte</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakbedekking</v>
       </c>
       <c r="B55" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -3599,10 +3599,10 @@
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/uitgesproken_gebrek</v>
       </c>
       <c r="E55" t="str">
-        <v>dakgebinte</v>
+        <v>dakbedekking</v>
       </c>
       <c r="F55" t="str">
-        <v>Gebrek aan de toestand van het dakgebinte</v>
+        <v>Gebrek aan de toestand van de dakbedekking</v>
       </c>
       <c r="G55" t="str">
         <v>null</v>
@@ -3629,13 +3629,13 @@
         <v>null</v>
       </c>
       <c r="O55" t="str">
-        <v>Dakgebinte</v>
+        <v>Dakbedekking</v>
       </c>
       <c r="P55" t="str">
         <v>http://www.eionet.europa.eu/gemet/theme/5</v>
       </c>
       <c r="Q55" t="str">
-        <v>https://data.omgeving.vlaanderen.be/ns/verwaarlozing#vertoont_gebrek_ivm_dakgebinte</v>
+        <v>https://data.omgeving.vlaanderen.be/ns/verwaarlozing#vertoont_gebrek_ivm_dakbedekking</v>
       </c>
       <c r="R55" t="str">
         <v>null</v>
@@ -3646,7 +3646,7 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakgoten</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakgebinte</v>
       </c>
       <c r="B56" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -3658,10 +3658,10 @@
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/uitgesproken_gebrek</v>
       </c>
       <c r="E56" t="str">
-        <v>dakgoten</v>
+        <v>dakgebinte</v>
       </c>
       <c r="F56" t="str">
-        <v>Gebrek aan de toestand van de dakgoten</v>
+        <v>Gebrek aan de toestand van het dakgebinte</v>
       </c>
       <c r="G56" t="str">
         <v>null</v>
@@ -3688,13 +3688,13 @@
         <v>null</v>
       </c>
       <c r="O56" t="str">
-        <v>Dakgoten</v>
+        <v>Dakgebinte</v>
       </c>
       <c r="P56" t="str">
         <v>http://www.eionet.europa.eu/gemet/theme/5</v>
       </c>
       <c r="Q56" t="str">
-        <v>https://data.omgeving.vlaanderen.be/ns/verwaarlozing#vertoont_gebrek_ivm_dakgoten</v>
+        <v>https://data.omgeving.vlaanderen.be/ns/verwaarlozing#vertoont_gebrek_ivm_dakgebinte</v>
       </c>
       <c r="R56" t="str">
         <v>null</v>
@@ -3705,7 +3705,7 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakgoten</v>
       </c>
       <c r="B57" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -3717,13 +3717,13 @@
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/uitgesproken_gebrek</v>
       </c>
       <c r="E57" t="str">
-        <v>gebouwonderdeel</v>
+        <v>dakgoten</v>
       </c>
       <c r="F57" t="str">
-        <v>Gebrek aan de toestand van een gebouwonderdeel</v>
+        <v>Gebrek aan de toestand van de dakgoten</v>
       </c>
       <c r="G57" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/uitgesproken_gebrek</v>
+        <v>null</v>
       </c>
       <c r="H57" t="str">
         <v>null</v>
@@ -3732,28 +3732,28 @@
         <v>null</v>
       </c>
       <c r="J57" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
       </c>
       <c r="K57" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
       </c>
       <c r="L57" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/buitenmuren|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/buitentimmerwerk|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakbedekking|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakgebinte|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakgoten|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/kroonlijst|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/liften|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/schoorstenen|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/trappen</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
       </c>
       <c r="M57" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/buitenmuren|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/buitentimmerwerk|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakbedekking|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakgebinte|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakgoten|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/kroonlijst|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/liften|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/schoorstenen|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/trappen</v>
+        <v>null</v>
       </c>
       <c r="N57" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/buitenmuren|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/buitentimmerwerk|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakbedekking|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakgebinte|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakgoten|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/kroonlijst|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/liften|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/schoorstenen|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/trappen</v>
+        <v>null</v>
       </c>
       <c r="O57" t="str">
-        <v>Gebrek aan de toestand van een gebouwonderdeel</v>
+        <v>Dakgoten</v>
       </c>
       <c r="P57" t="str">
         <v>http://www.eionet.europa.eu/gemet/theme/5</v>
       </c>
       <c r="Q57" t="str">
-        <v>https://data.omgeving.vlaanderen.be/ns/verwaarlozing#vertoont_gebrek_ivm_gebouwonderdeel</v>
+        <v>https://data.omgeving.vlaanderen.be/ns/verwaarlozing#vertoont_gebrek_ivm_dakgoten</v>
       </c>
       <c r="R57" t="str">
         <v>null</v>
@@ -3764,7 +3764,7 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/kroonlijst</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
       </c>
       <c r="B58" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -3776,13 +3776,13 @@
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/uitgesproken_gebrek</v>
       </c>
       <c r="E58" t="str">
-        <v>kroonlijst</v>
+        <v>gebouwonderdeel</v>
       </c>
       <c r="F58" t="str">
-        <v>Gebrek aan de toestand van de kroonlijst</v>
+        <v>Gebrek aan de toestand van een gebouwonderdeel</v>
       </c>
       <c r="G58" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/uitgesproken_gebrek</v>
       </c>
       <c r="H58" t="str">
         <v>null</v>
@@ -3791,28 +3791,28 @@
         <v>null</v>
       </c>
       <c r="J58" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
+        <v>null</v>
       </c>
       <c r="K58" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
+        <v>null</v>
       </c>
       <c r="L58" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/buitenmuren|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/buitentimmerwerk|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakbedekking|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakgebinte|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakgoten|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/kroonlijst|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/liften|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/schoorstenen|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/trappen</v>
       </c>
       <c r="M58" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/buitenmuren|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/buitentimmerwerk|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakbedekking|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakgebinte|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakgoten|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/kroonlijst|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/liften|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/schoorstenen|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/trappen</v>
       </c>
       <c r="N58" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/buitenmuren|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/buitentimmerwerk|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakbedekking|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakgebinte|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakgoten|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/kroonlijst|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/liften|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/schoorstenen|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/trappen</v>
       </c>
       <c r="O58" t="str">
-        <v>Kroonlijst</v>
+        <v>Gebrek aan de toestand van een gebouwonderdeel</v>
       </c>
       <c r="P58" t="str">
         <v>http://www.eionet.europa.eu/gemet/theme/5</v>
       </c>
       <c r="Q58" t="str">
-        <v>https://data.omgeving.vlaanderen.be/ns/verwaarlozing#vertoont_gebrek_ivm_kroonlijst</v>
+        <v>https://data.omgeving.vlaanderen.be/ns/verwaarlozing#vertoont_gebrek_ivm_gebouwonderdeel</v>
       </c>
       <c r="R58" t="str">
         <v>null</v>
@@ -3823,7 +3823,7 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/liften</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/kroonlijst</v>
       </c>
       <c r="B59" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -3835,10 +3835,10 @@
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/uitgesproken_gebrek</v>
       </c>
       <c r="E59" t="str">
-        <v>liften</v>
+        <v>kroonlijst</v>
       </c>
       <c r="F59" t="str">
-        <v>Gebrek aan de toestand van de liften</v>
+        <v>Gebrek aan de toestand van de kroonlijst</v>
       </c>
       <c r="G59" t="str">
         <v>null</v>
@@ -3865,13 +3865,13 @@
         <v>null</v>
       </c>
       <c r="O59" t="str">
-        <v>Liften</v>
+        <v>Kroonlijst</v>
       </c>
       <c r="P59" t="str">
         <v>http://www.eionet.europa.eu/gemet/theme/5</v>
       </c>
       <c r="Q59" t="str">
-        <v>https://data.omgeving.vlaanderen.be/ns/verwaarlozing#vertoont_gebrek_ivm_liften</v>
+        <v>https://data.omgeving.vlaanderen.be/ns/verwaarlozing#vertoont_gebrek_ivm_kroonlijst</v>
       </c>
       <c r="R59" t="str">
         <v>null</v>
@@ -3882,7 +3882,7 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/schoorstenen</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/liften</v>
       </c>
       <c r="B60" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -3894,10 +3894,10 @@
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/uitgesproken_gebrek</v>
       </c>
       <c r="E60" t="str">
-        <v>schoorstenen</v>
+        <v>liften</v>
       </c>
       <c r="F60" t="str">
-        <v>Gebrek aan de toestand van schoorstenen</v>
+        <v>Gebrek aan de toestand van de liften</v>
       </c>
       <c r="G60" t="str">
         <v>null</v>
@@ -3924,13 +3924,13 @@
         <v>null</v>
       </c>
       <c r="O60" t="str">
-        <v>Schoorstenen</v>
+        <v>Liften</v>
       </c>
       <c r="P60" t="str">
         <v>http://www.eionet.europa.eu/gemet/theme/5</v>
       </c>
       <c r="Q60" t="str">
-        <v>https://data.omgeving.vlaanderen.be/ns/verwaarlozing#vertoont_gebrek_ivm_schoorstenen</v>
+        <v>https://data.omgeving.vlaanderen.be/ns/verwaarlozing#vertoont_gebrek_ivm_liften</v>
       </c>
       <c r="R60" t="str">
         <v>null</v>
@@ -3941,7 +3941,7 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/stabiliteit</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/schoorstenen</v>
       </c>
       <c r="B61" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -3953,13 +3953,13 @@
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/uitgesproken_gebrek</v>
       </c>
       <c r="E61" t="str">
-        <v>stabiliteit</v>
+        <v>schoorstenen</v>
       </c>
       <c r="F61" t="str">
-        <v>Gebrek dat stabiliteit in het gedrang brengt</v>
+        <v>Gebrek aan de toestand van schoorstenen</v>
       </c>
       <c r="G61" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/uitgesproken_gebrek</v>
+        <v>null</v>
       </c>
       <c r="H61" t="str">
         <v>null</v>
@@ -3968,13 +3968,13 @@
         <v>null</v>
       </c>
       <c r="J61" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
       </c>
       <c r="K61" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
       </c>
       <c r="L61" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
       </c>
       <c r="M61" t="str">
         <v>null</v>
@@ -3983,13 +3983,13 @@
         <v>null</v>
       </c>
       <c r="O61" t="str">
-        <v>Gebrek dat stabiliteit in het gedrang brengt</v>
+        <v>Schoorstenen</v>
       </c>
       <c r="P61" t="str">
         <v>http://www.eionet.europa.eu/gemet/theme/5</v>
       </c>
       <c r="Q61" t="str">
-        <v>https://data.omgeving.vlaanderen.be/ns/verwaarlozing#vertoont_gebrek_ivm_stabiliteit</v>
+        <v>https://data.omgeving.vlaanderen.be/ns/verwaarlozing#vertoont_gebrek_ivm_schoorstenen</v>
       </c>
       <c r="R61" t="str">
         <v>null</v>
@@ -4000,7 +4000,7 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/trappen</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/stabiliteit</v>
       </c>
       <c r="B62" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -4012,13 +4012,13 @@
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/uitgesproken_gebrek</v>
       </c>
       <c r="E62" t="str">
-        <v>trappen</v>
+        <v>stabiliteit</v>
       </c>
       <c r="F62" t="str">
-        <v>Gebrek aan de toestand van de trappen</v>
+        <v>Gebrek dat stabiliteit in het gedrang brengt</v>
       </c>
       <c r="G62" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/uitgesproken_gebrek</v>
       </c>
       <c r="H62" t="str">
         <v>null</v>
@@ -4027,13 +4027,13 @@
         <v>null</v>
       </c>
       <c r="J62" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
+        <v>null</v>
       </c>
       <c r="K62" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
+        <v>null</v>
       </c>
       <c r="L62" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
+        <v>null</v>
       </c>
       <c r="M62" t="str">
         <v>null</v>
@@ -4042,13 +4042,13 @@
         <v>null</v>
       </c>
       <c r="O62" t="str">
-        <v>Trappen</v>
+        <v>Gebrek dat stabiliteit in het gedrang brengt</v>
       </c>
       <c r="P62" t="str">
         <v>http://www.eionet.europa.eu/gemet/theme/5</v>
       </c>
       <c r="Q62" t="str">
-        <v>https://data.omgeving.vlaanderen.be/ns/verwaarlozing#vertoont_gebrek_ivm_trappen</v>
+        <v>https://data.omgeving.vlaanderen.be/ns/verwaarlozing#vertoont_gebrek_ivm_stabiliteit</v>
       </c>
       <c r="R62" t="str">
         <v>null</v>
@@ -4059,7 +4059,7 @@
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/veiligheid</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/trappen</v>
       </c>
       <c r="B63" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -4071,13 +4071,13 @@
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/uitgesproken_gebrek</v>
       </c>
       <c r="E63" t="str">
-        <v>veiligheid</v>
+        <v>trappen</v>
       </c>
       <c r="F63" t="str">
-        <v>Gebrek dat veiligheid in het gedrang brengt</v>
+        <v>Gebrek aan de toestand van de trappen</v>
       </c>
       <c r="G63" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/uitgesproken_gebrek</v>
+        <v>null</v>
       </c>
       <c r="H63" t="str">
         <v>null</v>
@@ -4086,13 +4086,13 @@
         <v>null</v>
       </c>
       <c r="J63" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
       </c>
       <c r="K63" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
       </c>
       <c r="L63" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
       </c>
       <c r="M63" t="str">
         <v>null</v>
@@ -4101,13 +4101,13 @@
         <v>null</v>
       </c>
       <c r="O63" t="str">
-        <v>Gebrek dat veiligheid in het gedrang brengt</v>
+        <v>Trappen</v>
       </c>
       <c r="P63" t="str">
         <v>http://www.eionet.europa.eu/gemet/theme/5</v>
       </c>
       <c r="Q63" t="str">
-        <v>https://data.omgeving.vlaanderen.be/ns/verwaarlozing#vertoont_gebrek_ivm_veiligheid</v>
+        <v>https://data.omgeving.vlaanderen.be/ns/verwaarlozing#vertoont_gebrek_ivm_trappen</v>
       </c>
       <c r="R63" t="str">
         <v>null</v>
@@ -4118,7 +4118,7 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/vochtindringing</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/veiligheid</v>
       </c>
       <c r="B64" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -4130,10 +4130,10 @@
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/uitgesproken_gebrek</v>
       </c>
       <c r="E64" t="str">
-        <v>vochtindringing</v>
+        <v>veiligheid</v>
       </c>
       <c r="F64" t="str">
-        <v>Gebrek dat leidt tot vochtindringing</v>
+        <v>Gebrek dat veiligheid in het gedrang brengt</v>
       </c>
       <c r="G64" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/uitgesproken_gebrek</v>
@@ -4160,13 +4160,13 @@
         <v>null</v>
       </c>
       <c r="O64" t="str">
-        <v>Gebrek dat leidt tot vochtindringing</v>
+        <v>Gebrek dat veiligheid in het gedrang brengt</v>
       </c>
       <c r="P64" t="str">
         <v>http://www.eionet.europa.eu/gemet/theme/5</v>
       </c>
       <c r="Q64" t="str">
-        <v>https://data.omgeving.vlaanderen.be/ns/verwaarlozing#vertoont_gebrek_ivm_vochtindringing</v>
+        <v>https://data.omgeving.vlaanderen.be/ns/verwaarlozing#vertoont_gebrek_ivm_veiligheid</v>
       </c>
       <c r="R64" t="str">
         <v>null</v>
@@ -4177,31 +4177,31 @@
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/aanvraag_opschorting_heffing_reden</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/vochtindringing</v>
       </c>
       <c r="B65" t="str">
-        <v>http://www.w3.org/2004/02/skos/core#ConceptScheme</v>
+        <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C65" t="str">
         <v>null</v>
       </c>
       <c r="D65" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/uitgesproken_gebrek</v>
       </c>
       <c r="E65" t="str">
-        <v>cs_aanvraag_opschorting_heffing_reden</v>
+        <v>vochtindringing</v>
       </c>
       <c r="F65" t="str">
-        <v>Conceptschema over reden voor een procedure aanvraag opschorting heffing</v>
+        <v>Gebrek dat leidt tot vochtindringing</v>
       </c>
       <c r="G65" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/uitgesproken_gebrek</v>
       </c>
       <c r="H65" t="str">
-        <v>Conceptschema over reden voor een procedure aanvraag opschorting heffing</v>
+        <v>null</v>
       </c>
       <c r="I65" t="str">
-        <v>Conceptschema over reden voor een procedure aanvraag opschorting heffing</v>
+        <v>null</v>
       </c>
       <c r="J65" t="str">
         <v>null</v>
@@ -4219,24 +4219,24 @@
         <v>null</v>
       </c>
       <c r="O65" t="str">
-        <v>null</v>
+        <v>Gebrek dat leidt tot vochtindringing</v>
       </c>
       <c r="P65" t="str">
-        <v>null</v>
+        <v>http://www.eionet.europa.eu/gemet/theme/5</v>
       </c>
       <c r="Q65" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/ns/verwaarlozing#vertoont_gebrek_ivm_vochtindringing</v>
       </c>
       <c r="R65" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/dataset/codelijst-verwaarlozing</v>
+        <v>null</v>
       </c>
       <c r="S65" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/aanvraag_opschorting_heffing_reden/bodemsaneringsproject|https://data.omgeving.vlaanderen.be/id/concept/leegstand/aanvraag_opschorting_heffing_reden/brownfieldconvenant|https://data.omgeving.vlaanderen.be/id/concept/leegstand/aanvraag_opschorting_heffing_reden/leegstaand_niet_verwaarloosd|https://data.omgeving.vlaanderen.be/id/concept/leegstand/aanvraag_opschorting_heffing_reden/nieuwe_eigenaars|https://data.omgeving.vlaanderen.be/id/concept/leegstand/aanvraag_opschorting_heffing_reden/verlenging_bij_vernieuwing|https://data.omgeving.vlaanderen.be/id/concept/leegstand/aanvraag_opschorting_heffing_reden/vernieuwing</v>
+        <v>null</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/beslissing</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/aanvraag_opschorting_heffing_reden</v>
       </c>
       <c r="B66" t="str">
         <v>http://www.w3.org/2004/02/skos/core#ConceptScheme</v>
@@ -4248,19 +4248,19 @@
         <v>null</v>
       </c>
       <c r="E66" t="str">
-        <v>cs_beslissing</v>
+        <v>cs_aanvraag_opschorting_heffing_reden</v>
       </c>
       <c r="F66" t="str">
-        <v>Conceptschema over beslissingen die genomen kunnen worden binnen procedures in het kader van leegstaande en verwaarloosde bedrijfsruimten.</v>
+        <v>Conceptschema over reden voor een procedure aanvraag opschorting heffing</v>
       </c>
       <c r="G66" t="str">
         <v>null</v>
       </c>
       <c r="H66" t="str">
-        <v>Conceptschema over beslissingen die genomen kunnen worden binnen procedures in het kader van leegstaande en verwaarloosde bedrijfsruimten.</v>
+        <v>Conceptschema over reden voor een procedure aanvraag opschorting heffing</v>
       </c>
       <c r="I66" t="str">
-        <v>Conceptschema over beslissingen die genomen kunnen worden binnen procedures in het kader van leegstaande en verwaarloosde bedrijfsruimten.</v>
+        <v>Conceptschema over reden voor een procedure aanvraag opschorting heffing</v>
       </c>
       <c r="J66" t="str">
         <v>null</v>
@@ -4290,12 +4290,12 @@
         <v>https://data.omgeving.vlaanderen.be/id/dataset/codelijst-verwaarlozing</v>
       </c>
       <c r="S66" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/aanvraag_opschorting_heffing_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/aanvraag_opschorting_heffing_niet_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/aanvraag_schrapping_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/aanvraag_schrapping_niet_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/beroep_tegen_registratie_ingewilligd|https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/beroep_tegen_registratie_onontvankelijk_verklaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/beroep_tegen_registratie_verworpen|https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/geregistreerd_in_inventaris|https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/geschrapt_uit_inventaris|https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/heffing_opgeschort|https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/niet_geregistreerd_in_inventaris|https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/registratie_ingetrokken</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/aanvraag_opschorting_heffing_reden/bodemsaneringsproject|https://data.omgeving.vlaanderen.be/id/concept/leegstand/aanvraag_opschorting_heffing_reden/brownfieldconvenant|https://data.omgeving.vlaanderen.be/id/concept/leegstand/aanvraag_opschorting_heffing_reden/leegstaand_niet_verwaarloosd|https://data.omgeving.vlaanderen.be/id/concept/leegstand/aanvraag_opschorting_heffing_reden/nieuwe_eigenaars|https://data.omgeving.vlaanderen.be/id/concept/leegstand/aanvraag_opschorting_heffing_reden/verlenging_bij_vernieuwing|https://data.omgeving.vlaanderen.be/id/concept/leegstand/aanvraag_opschorting_heffing_reden/vernieuwing</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/procedure</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/beslissing</v>
       </c>
       <c r="B67" t="str">
         <v>http://www.w3.org/2004/02/skos/core#ConceptScheme</v>
@@ -4307,19 +4307,19 @@
         <v>null</v>
       </c>
       <c r="E67" t="str">
-        <v>cs_procedure</v>
+        <v>cs_beslissing</v>
       </c>
       <c r="F67" t="str">
-        <v>Conceptschema over procedures in het kader van leegstaande en verwaarloosde bedrijfsruimten.</v>
+        <v>Conceptschema over beslissingen die genomen kunnen worden binnen procedures in het kader van leegstaande en verwaarloosde bedrijfsruimten.</v>
       </c>
       <c r="G67" t="str">
         <v>null</v>
       </c>
       <c r="H67" t="str">
-        <v>Conceptschema over procedures in het kader van leegstaande en verwaarloosde bedrijfsruimten.</v>
+        <v>Conceptschema over beslissingen die genomen kunnen worden binnen procedures in het kader van leegstaande en verwaarloosde bedrijfsruimten.</v>
       </c>
       <c r="I67" t="str">
-        <v>Conceptschema over procedures in het kader van leegstaande en verwaarloosde bedrijfsruimten.</v>
+        <v>Conceptschema over beslissingen die genomen kunnen worden binnen procedures in het kader van leegstaande en verwaarloosde bedrijfsruimten.</v>
       </c>
       <c r="J67" t="str">
         <v>null</v>
@@ -4349,12 +4349,12 @@
         <v>https://data.omgeving.vlaanderen.be/id/dataset/codelijst-verwaarlozing</v>
       </c>
       <c r="S67" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/procedure/aanvraag_opschorting_heffing|https://data.omgeving.vlaanderen.be/id/concept/leegstand/procedure/aanvraag_schrapping|https://data.omgeving.vlaanderen.be/id/concept/leegstand/procedure/beroep_tegen_registratie|https://data.omgeving.vlaanderen.be/id/concept/leegstand/procedure/registreren</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/aanvraag_opschorting_heffing_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/aanvraag_opschorting_heffing_niet_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/aanvraag_schrapping_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/aanvraag_schrapping_niet_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/beroep_tegen_registratie_ingewilligd|https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/beroep_tegen_registratie_onontvankelijk_verklaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/beroep_tegen_registratie_verworpen|https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/geregistreerd_in_inventaris|https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/geschrapt_uit_inventaris|https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/heffing_opgeschort|https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/niet_geregistreerd_in_inventaris|https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/registratie_ingetrokken</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/rol</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/procedure</v>
       </c>
       <c r="B68" t="str">
         <v>http://www.w3.org/2004/02/skos/core#ConceptScheme</v>
@@ -4366,19 +4366,19 @@
         <v>null</v>
       </c>
       <c r="E68" t="str">
-        <v>cs_rol</v>
+        <v>cs_procedure</v>
       </c>
       <c r="F68" t="str">
-        <v>Conceptschema over rollen van agenten binnen procedures in het kader van leegstaande en verwaarloosde bedrijfsruimten.</v>
+        <v>Conceptschema over procedures in het kader van leegstaande en verwaarloosde bedrijfsruimten.</v>
       </c>
       <c r="G68" t="str">
         <v>null</v>
       </c>
       <c r="H68" t="str">
-        <v>Conceptschema over rollen van agenten binnen procedures in het kader van leegstaande en verwaarloosde bedrijfsruimten.</v>
+        <v>Conceptschema over procedures in het kader van leegstaande en verwaarloosde bedrijfsruimten.</v>
       </c>
       <c r="I68" t="str">
-        <v>Conceptschema over rollen van agenten binnen procedures in het kader van leegstaande en verwaarloosde bedrijfsruimten.</v>
+        <v>Conceptschema over procedures in het kader van leegstaande en verwaarloosde bedrijfsruimten.</v>
       </c>
       <c r="J68" t="str">
         <v>null</v>
@@ -4408,12 +4408,12 @@
         <v>https://data.omgeving.vlaanderen.be/id/dataset/codelijst-verwaarlozing</v>
       </c>
       <c r="S68" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/rol/curator|https://data.omgeving.vlaanderen.be/id/concept/leegstand/rol/eigenaar|https://data.omgeving.vlaanderen.be/id/concept/leegstand/rol/instrumenterend_ambtenaar|https://data.omgeving.vlaanderen.be/id/concept/leegstand/rol/raadsman</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/procedure/aanvraag_opschorting_heffing|https://data.omgeving.vlaanderen.be/id/concept/leegstand/procedure/aanvraag_schrapping|https://data.omgeving.vlaanderen.be/id/concept/leegstand/procedure/beroep_tegen_registratie|https://data.omgeving.vlaanderen.be/id/concept/leegstand/procedure/registreren</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/rol</v>
       </c>
       <c r="B69" t="str">
         <v>http://www.w3.org/2004/02/skos/core#ConceptScheme</v>
@@ -4425,19 +4425,19 @@
         <v>null</v>
       </c>
       <c r="E69" t="str">
-        <v>cs_stuk</v>
+        <v>cs_rol</v>
       </c>
       <c r="F69" t="str">
-        <v>Conceptschema over stukken in het kader van leegstaande en verwaarloosde bedrijfsruimten.</v>
+        <v>Conceptschema over rollen van agenten binnen procedures in het kader van leegstaande en verwaarloosde bedrijfsruimten.</v>
       </c>
       <c r="G69" t="str">
         <v>null</v>
       </c>
       <c r="H69" t="str">
-        <v>Conceptschema over stukken in het kader van leegstaande en verwaarloosde bedrijfsruimten.</v>
+        <v>Conceptschema over rollen van agenten binnen procedures in het kader van leegstaande en verwaarloosde bedrijfsruimten.</v>
       </c>
       <c r="I69" t="str">
-        <v>Conceptschema over stukken in het kader van leegstaande en verwaarloosde bedrijfsruimten.</v>
+        <v>Conceptschema over rollen van agenten binnen procedures in het kader van leegstaande en verwaarloosde bedrijfsruimten.</v>
       </c>
       <c r="J69" t="str">
         <v>null</v>
@@ -4467,12 +4467,12 @@
         <v>https://data.omgeving.vlaanderen.be/id/dataset/codelijst-verwaarlozing</v>
       </c>
       <c r="S69" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/stavingsstuk|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/procedurestuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/rol/bewindvoerder|https://data.omgeving.vlaanderen.be/id/concept/leegstand/rol/curator|https://data.omgeving.vlaanderen.be/id/concept/leegstand/rol/eigenaar|https://data.omgeving.vlaanderen.be/id/concept/leegstand/rol/instrumenterend_ambtenaar|https://data.omgeving.vlaanderen.be/id/concept/leegstand/rol/raadsman</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/uitgesproken_gebrek</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="B70" t="str">
         <v>http://www.w3.org/2004/02/skos/core#ConceptScheme</v>
@@ -4484,19 +4484,19 @@
         <v>null</v>
       </c>
       <c r="E70" t="str">
-        <v>cs_uitgesproken_gebrek</v>
+        <v>cs_stuk</v>
       </c>
       <c r="F70" t="str">
-        <v>Conceptschema over kenmerken van verwaarlozing aan gebouwen.</v>
+        <v>Conceptschema over stukken in het kader van leegstaande en verwaarloosde bedrijfsruimten.</v>
       </c>
       <c r="G70" t="str">
         <v>null</v>
       </c>
       <c r="H70" t="str">
-        <v>Het vertonen van uitgesproken gebreken van algemene of beperkte omvang van bedrijfsverwaarlozing. De Vlaamse regering bepaalt de gebreken van algemene en beperkte omvang, alsook de criteria voor de beoordeling van de gebreken en de minimumnorm van de te vertonen gebreken om een bedrijfsruimte al dan niet als geheel of gedeeltelijk verwaarloosd te beschouwen;</v>
+        <v>Conceptschema over stukken in het kader van leegstaande en verwaarloosde bedrijfsruimten.</v>
       </c>
       <c r="I70" t="str">
-        <v>Het vertonen van uitgesproken gebreken van algemene of beperkte omvang van bedrijfsverwaarlozing. De Vlaamse regering bepaalt de gebreken van algemene en beperkte omvang, alsook de criteria voor de beoordeling van de gebreken en de minimumnorm van de te vertonen gebreken om een bedrijfsruimte al dan niet als geheel of gedeeltelijk verwaarloosd te beschouwen;</v>
+        <v>Conceptschema over stukken in het kader van leegstaande en verwaarloosde bedrijfsruimten.</v>
       </c>
       <c r="J70" t="str">
         <v>null</v>
@@ -4517,7 +4517,7 @@
         <v>null</v>
       </c>
       <c r="P70" t="str">
-        <v>http://www.eionet.europa.eu/gemet/theme/5</v>
+        <v>null</v>
       </c>
       <c r="Q70" t="str">
         <v>null</v>
@@ -4526,12 +4526,71 @@
         <v>https://data.omgeving.vlaanderen.be/id/dataset/codelijst-verwaarlozing</v>
       </c>
       <c r="S70" t="str">
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/stavingsstuk|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/procedurestuk</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/uitgesproken_gebrek</v>
+      </c>
+      <c r="B71" t="str">
+        <v>http://www.w3.org/2004/02/skos/core#ConceptScheme</v>
+      </c>
+      <c r="C71" t="str">
+        <v>null</v>
+      </c>
+      <c r="D71" t="str">
+        <v>null</v>
+      </c>
+      <c r="E71" t="str">
+        <v>cs_uitgesproken_gebrek</v>
+      </c>
+      <c r="F71" t="str">
+        <v>Conceptschema over kenmerken van verwaarlozing aan gebouwen.</v>
+      </c>
+      <c r="G71" t="str">
+        <v>null</v>
+      </c>
+      <c r="H71" t="str">
+        <v>Het vertonen van uitgesproken gebreken van algemene of beperkte omvang van bedrijfsverwaarlozing. De Vlaamse regering bepaalt de gebreken van algemene en beperkte omvang, alsook de criteria voor de beoordeling van de gebreken en de minimumnorm van de te vertonen gebreken om een bedrijfsruimte al dan niet als geheel of gedeeltelijk verwaarloosd te beschouwen;</v>
+      </c>
+      <c r="I71" t="str">
+        <v>Het vertonen van uitgesproken gebreken van algemene of beperkte omvang van bedrijfsverwaarlozing. De Vlaamse regering bepaalt de gebreken van algemene en beperkte omvang, alsook de criteria voor de beoordeling van de gebreken en de minimumnorm van de te vertonen gebreken om een bedrijfsruimte al dan niet als geheel of gedeeltelijk verwaarloosd te beschouwen;</v>
+      </c>
+      <c r="J71" t="str">
+        <v>null</v>
+      </c>
+      <c r="K71" t="str">
+        <v>null</v>
+      </c>
+      <c r="L71" t="str">
+        <v>null</v>
+      </c>
+      <c r="M71" t="str">
+        <v>null</v>
+      </c>
+      <c r="N71" t="str">
+        <v>null</v>
+      </c>
+      <c r="O71" t="str">
+        <v>null</v>
+      </c>
+      <c r="P71" t="str">
+        <v>http://www.eionet.europa.eu/gemet/theme/5</v>
+      </c>
+      <c r="Q71" t="str">
+        <v>null</v>
+      </c>
+      <c r="R71" t="str">
+        <v>https://data.omgeving.vlaanderen.be/id/dataset/codelijst-verwaarlozing</v>
+      </c>
+      <c r="S71" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/stabiliteit|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/veiligheid|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/vochtindringing</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S70"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S71"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
LVBR-386: Hernoemen schrapping naar reden_van_verwijderen_uit_inventaris
</commit_message>
<xml_diff>
--- a/src/main/resources/be/vlaanderen/omgeving/data/id/conceptscheme/verwaarlozing/verwaarlozing.xlsx
+++ b/src/main/resources/be/vlaanderen/omgeving/data/id/conceptscheme/verwaarlozing/verwaarlozing.xlsx
@@ -2053,25 +2053,25 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/schrapping/benutting_meer_dan_vijftig_percent</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_aanvaard</v>
       </c>
       <c r="B29" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C29" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/aanvraag_opschorting_heffing_aanvaard</v>
       </c>
       <c r="D29" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/schrapping</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E29" t="str">
-        <v>+50%</v>
+        <v>OPSCH_ANVRD</v>
       </c>
       <c r="F29" t="str">
-        <v>Benutting van meer dan 50% conform de vergunde bestemming van het gebouw</v>
+        <v>Opschorting aanvaard</v>
       </c>
       <c r="G29" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/schrapping</v>
+        <v>null</v>
       </c>
       <c r="H29" t="str">
         <v>null</v>
@@ -2080,13 +2080,13 @@
         <v>null</v>
       </c>
       <c r="J29" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
       </c>
       <c r="K29" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
       </c>
       <c r="L29" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
       </c>
       <c r="M29" t="str">
         <v>null</v>
@@ -2112,25 +2112,25 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/schrapping/functiewijziging</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_aanvaard_begeleidende_brief</v>
       </c>
       <c r="B30" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C30" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_aanvaard</v>
       </c>
       <c r="D30" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/schrapping</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E30" t="str">
-        <v>functiewijziging</v>
+        <v>OPSCH_ANVRD_BEG_BRIEF</v>
       </c>
       <c r="F30" t="str">
-        <v>Functiewijziging doorgevoerd</v>
+        <v>Begeleidende brief bij opschorting aanvaard</v>
       </c>
       <c r="G30" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/schrapping</v>
+        <v>null</v>
       </c>
       <c r="H30" t="str">
         <v>null</v>
@@ -2139,13 +2139,13 @@
         <v>null</v>
       </c>
       <c r="J30" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
       </c>
       <c r="K30" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
       </c>
       <c r="L30" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
       </c>
       <c r="M30" t="str">
         <v>null</v>
@@ -2171,25 +2171,25 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/schrapping/gesloopt</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_niet_aanvaard</v>
       </c>
       <c r="B31" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C31" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/aanvraag_opschorting_heffing_niet_aanvaard</v>
       </c>
       <c r="D31" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/schrapping</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E31" t="str">
-        <v>gesloopt</v>
+        <v>OPSCH_NANVRD</v>
       </c>
       <c r="F31" t="str">
-        <v>De bedrijfsruimte is gesloopt</v>
+        <v>Opschorting niet aanvaard</v>
       </c>
       <c r="G31" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/schrapping</v>
+        <v>null</v>
       </c>
       <c r="H31" t="str">
         <v>null</v>
@@ -2198,13 +2198,13 @@
         <v>null</v>
       </c>
       <c r="J31" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
       </c>
       <c r="K31" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
       </c>
       <c r="L31" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
       </c>
       <c r="M31" t="str">
         <v>null</v>
@@ -2230,25 +2230,25 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/schrapping/heffing</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_niet_aanvaard_begeleidende_brief</v>
       </c>
       <c r="B32" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C32" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_niet_aanvaard</v>
       </c>
       <c r="D32" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/schrapping</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E32" t="str">
-        <v>heffing</v>
+        <v>OPSCH_NANVRD_BEG_BRIEF</v>
       </c>
       <c r="F32" t="str">
-        <v>Procedure heffing</v>
+        <v>Begeleidende brief bij opschorting niet aanvaard</v>
       </c>
       <c r="G32" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/schrapping</v>
+        <v>null</v>
       </c>
       <c r="H32" t="str">
         <v>null</v>
@@ -2257,13 +2257,13 @@
         <v>null</v>
       </c>
       <c r="J32" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
       </c>
       <c r="K32" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
       </c>
       <c r="L32" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
       </c>
       <c r="M32" t="str">
         <v>null</v>
@@ -2289,25 +2289,25 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/schrapping/nieuwe_invulling</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_aanvaard</v>
       </c>
       <c r="B33" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C33" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/aanvraag_schrapping_aanvaard</v>
       </c>
       <c r="D33" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/schrapping</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E33" t="str">
-        <v>nieuwe_invulling</v>
+        <v>SCHR_ANVRD</v>
       </c>
       <c r="F33" t="str">
-        <v>Nieuwe invulling gegeven conform de vergunde bestemming</v>
+        <v>Schrapping aanvaard</v>
       </c>
       <c r="G33" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/schrapping</v>
+        <v>null</v>
       </c>
       <c r="H33" t="str">
         <v>null</v>
@@ -2316,13 +2316,13 @@
         <v>null</v>
       </c>
       <c r="J33" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
       </c>
       <c r="K33" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
       </c>
       <c r="L33" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
       </c>
       <c r="M33" t="str">
         <v>null</v>
@@ -2348,25 +2348,25 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/schrapping/onteigening</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_aanvaard_begeleidende_brief</v>
       </c>
       <c r="B34" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C34" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_aanvaard</v>
       </c>
       <c r="D34" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/schrapping</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E34" t="str">
-        <v>onteigening</v>
+        <v>SCHR_ANVRD_BEG_BRIEF</v>
       </c>
       <c r="F34" t="str">
-        <v>Er is een onteigening</v>
+        <v>Begeleidende brief bij schrapping aanvaard</v>
       </c>
       <c r="G34" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/schrapping</v>
+        <v>null</v>
       </c>
       <c r="H34" t="str">
         <v>null</v>
@@ -2375,13 +2375,13 @@
         <v>null</v>
       </c>
       <c r="J34" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
       </c>
       <c r="K34" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
       </c>
       <c r="L34" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
       </c>
       <c r="M34" t="str">
         <v>null</v>
@@ -2407,25 +2407,25 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/schrapping/opgeheven</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_niet_aanvaard</v>
       </c>
       <c r="B35" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C35" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/aanvraag_schrapping_niet_aanvaard</v>
       </c>
       <c r="D35" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/schrapping</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E35" t="str">
-        <v>opgeheven</v>
+        <v>SCHR_NANVRD</v>
       </c>
       <c r="F35" t="str">
-        <v>Verwaarlozing is opgeheven</v>
+        <v>Schrapping niet aanvaard</v>
       </c>
       <c r="G35" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/schrapping</v>
+        <v>null</v>
       </c>
       <c r="H35" t="str">
         <v>null</v>
@@ -2434,13 +2434,13 @@
         <v>null</v>
       </c>
       <c r="J35" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
       </c>
       <c r="K35" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
       </c>
       <c r="L35" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
       </c>
       <c r="M35" t="str">
         <v>null</v>
@@ -2466,25 +2466,25 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/schrapping/rechtbank</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_niet_aanvaard_begeleidende_brief</v>
       </c>
       <c r="B36" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C36" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_niet_aanvaard</v>
       </c>
       <c r="D36" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/schrapping</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E36" t="str">
-        <v>rechtbank</v>
+        <v>SCHR_NANVRD_BEG_BRIEF</v>
       </c>
       <c r="F36" t="str">
-        <v>Procedure rechtbank</v>
+        <v>Begeleidende brief bij schrapping niet aanvaard</v>
       </c>
       <c r="G36" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/schrapping</v>
+        <v>null</v>
       </c>
       <c r="H36" t="str">
         <v>null</v>
@@ -2493,13 +2493,13 @@
         <v>null</v>
       </c>
       <c r="J36" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
       </c>
       <c r="K36" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
       </c>
       <c r="L36" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
       </c>
       <c r="M36" t="str">
         <v>null</v>
@@ -2525,22 +2525,22 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_aanvaard</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_ingewilligd</v>
       </c>
       <c r="B37" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C37" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/aanvraag_opschorting_heffing_aanvaard</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/beroep_tegen_registratie_ingewilligd</v>
       </c>
       <c r="D37" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E37" t="str">
-        <v>OPSCH_ANVRD</v>
+        <v>BER_INGWD</v>
       </c>
       <c r="F37" t="str">
-        <v>Opschorting aanvaard</v>
+        <v>Beroep ingewilligd</v>
       </c>
       <c r="G37" t="str">
         <v>null</v>
@@ -2584,22 +2584,22 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_aanvaard_begeleidende_brief</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_ingewilligd_begeleidende_brief</v>
       </c>
       <c r="B38" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C38" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_aanvaard</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_ingewilligd</v>
       </c>
       <c r="D38" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E38" t="str">
-        <v>OPSCH_ANVRD_BEG_BRIEF</v>
+        <v>BER_INGWD_BEG_BRIEF</v>
       </c>
       <c r="F38" t="str">
-        <v>Begeleidende brief bij opschorting aanvaard</v>
+        <v>Begeleidende brief bij beroep ingewilligd</v>
       </c>
       <c r="G38" t="str">
         <v>null</v>
@@ -2643,22 +2643,22 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_niet_aanvaard</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_onontvankelijk_verklaard</v>
       </c>
       <c r="B39" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C39" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/aanvraag_opschorting_heffing_niet_aanvaard</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/beroep_tegen_registratie_onontvankelijk_verklaard</v>
       </c>
       <c r="D39" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E39" t="str">
-        <v>OPSCH_NANVRD</v>
+        <v>BER_ON</v>
       </c>
       <c r="F39" t="str">
-        <v>Opschorting niet aanvaard</v>
+        <v>Beroep onontvankelijk verklaard</v>
       </c>
       <c r="G39" t="str">
         <v>null</v>
@@ -2702,22 +2702,22 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_niet_aanvaard_begeleidende_brief</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_onontvankelijk_verklaard_begeleidende_brief</v>
       </c>
       <c r="B40" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C40" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_niet_aanvaard</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_onontvankelijk_verklaard</v>
       </c>
       <c r="D40" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E40" t="str">
-        <v>OPSCH_NANVRD_BEG_BRIEF</v>
+        <v>BER_ON_BEG_BRIEF</v>
       </c>
       <c r="F40" t="str">
-        <v>Begeleidende brief bij opschorting niet aanvaard</v>
+        <v>Begeleidende brief bij beroep onontvankelijk verklaard</v>
       </c>
       <c r="G40" t="str">
         <v>null</v>
@@ -2761,22 +2761,22 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_aanvaard</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_verworpen</v>
       </c>
       <c r="B41" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C41" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/aanvraag_schrapping_aanvaard</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/beroep_tegen_registratie_verworpen</v>
       </c>
       <c r="D41" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E41" t="str">
-        <v>SCHR_ANVRD</v>
+        <v>BER_VERWN</v>
       </c>
       <c r="F41" t="str">
-        <v>Schrapping aanvaard</v>
+        <v>Beroep verworpen</v>
       </c>
       <c r="G41" t="str">
         <v>null</v>
@@ -2820,22 +2820,22 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_aanvaard_begeleidende_brief</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_verworpen_begeleidende_brief</v>
       </c>
       <c r="B42" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C42" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_aanvaard</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_verworpen</v>
       </c>
       <c r="D42" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E42" t="str">
-        <v>SCHR_ANVRD_BEG_BRIEF</v>
+        <v>BER_VERWN_BEG_BRIEF</v>
       </c>
       <c r="F42" t="str">
-        <v>Begeleidende brief bij schrapping aanvaard</v>
+        <v>Begeleidende brief bij beroep verworpen</v>
       </c>
       <c r="G42" t="str">
         <v>null</v>
@@ -2879,25 +2879,25 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_niet_aanvaard</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
       </c>
       <c r="B43" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C43" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/aanvraag_schrapping_niet_aanvaard</v>
+        <v>null</v>
       </c>
       <c r="D43" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E43" t="str">
-        <v>SCHR_NANVRD</v>
+        <v>beslissingsstuk</v>
       </c>
       <c r="F43" t="str">
-        <v>Schrapping niet aanvaard</v>
+        <v>Stuk dat voortkomt uit een beslissing</v>
       </c>
       <c r="G43" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="H43" t="str">
         <v>null</v>
@@ -2906,19 +2906,19 @@
         <v>null</v>
       </c>
       <c r="J43" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
+        <v>null</v>
       </c>
       <c r="K43" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
+        <v>null</v>
       </c>
       <c r="L43" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_niet_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_niet_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_niet_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_niet_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_ingewilligd|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_ingewilligd_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_onontvankelijk_verklaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_onontvankelijk_verklaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_verworpen|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_verworpen_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/registratieattest|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/registratieattest_begeleidende_brief</v>
       </c>
       <c r="M43" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_niet_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_niet_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_niet_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_niet_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_ingewilligd|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_ingewilligd_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_onontvankelijk_verklaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_onontvankelijk_verklaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_verworpen|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_verworpen_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/registratieattest|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/registratieattest_begeleidende_brief</v>
       </c>
       <c r="N43" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_niet_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_niet_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_niet_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_niet_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_ingewilligd|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_ingewilligd_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_onontvankelijk_verklaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_onontvankelijk_verklaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_verworpen|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_verworpen_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/registratieattest|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/registratieattest_begeleidende_brief</v>
       </c>
       <c r="O43" t="str">
         <v>null</v>
@@ -2938,22 +2938,22 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_niet_aanvaard_begeleidende_brief</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/foto</v>
       </c>
       <c r="B44" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C44" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_niet_aanvaard</v>
+        <v>null</v>
       </c>
       <c r="D44" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E44" t="str">
-        <v>SCHR_NANVRD_BEG_BRIEF</v>
+        <v>FOTO</v>
       </c>
       <c r="F44" t="str">
-        <v>Begeleidende brief bij schrapping niet aanvaard</v>
+        <v>Foto</v>
       </c>
       <c r="G44" t="str">
         <v>null</v>
@@ -2965,13 +2965,13 @@
         <v>null</v>
       </c>
       <c r="J44" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/stavingsstuk</v>
       </c>
       <c r="K44" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/stavingsstuk</v>
       </c>
       <c r="L44" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/stavingsstuk</v>
       </c>
       <c r="M44" t="str">
         <v>null</v>
@@ -2997,22 +2997,22 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_ingewilligd</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/inkomend_procedurestuk</v>
       </c>
       <c r="B45" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C45" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/beroep_tegen_registratie_ingewilligd</v>
+        <v>null</v>
       </c>
       <c r="D45" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E45" t="str">
-        <v>BER_INGWD</v>
+        <v>INKOMEND_PROCEDURESTUK</v>
       </c>
       <c r="F45" t="str">
-        <v>Beroep ingewilligd</v>
+        <v>Inkomend procedurestuk</v>
       </c>
       <c r="G45" t="str">
         <v>null</v>
@@ -3024,13 +3024,13 @@
         <v>null</v>
       </c>
       <c r="J45" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/procedurestuk</v>
       </c>
       <c r="K45" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/procedurestuk</v>
       </c>
       <c r="L45" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/procedurestuk</v>
       </c>
       <c r="M45" t="str">
         <v>null</v>
@@ -3056,25 +3056,25 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_ingewilligd_begeleidende_brief</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/procedurestuk</v>
       </c>
       <c r="B46" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C46" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_ingewilligd</v>
+        <v>null</v>
       </c>
       <c r="D46" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E46" t="str">
-        <v>BER_INGWD_BEG_BRIEF</v>
+        <v>procedurestuk</v>
       </c>
       <c r="F46" t="str">
-        <v>Begeleidende brief bij beroep ingewilligd</v>
+        <v>Stuk gerelateerd aan een procedure</v>
       </c>
       <c r="G46" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="H46" t="str">
         <v>null</v>
@@ -3083,19 +3083,19 @@
         <v>null</v>
       </c>
       <c r="J46" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
+        <v>null</v>
       </c>
       <c r="K46" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
+        <v>null</v>
       </c>
       <c r="L46" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/inkomend_procedurestuk|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/retour_afzender_procedurestuk</v>
       </c>
       <c r="M46" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/inkomend_procedurestuk|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/retour_afzender_procedurestuk</v>
       </c>
       <c r="N46" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/inkomend_procedurestuk|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/retour_afzender_procedurestuk</v>
       </c>
       <c r="O46" t="str">
         <v>null</v>
@@ -3115,22 +3115,22 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_onontvankelijk_verklaard</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/registratieattest</v>
       </c>
       <c r="B47" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C47" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/beroep_tegen_registratie_onontvankelijk_verklaard</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/geregistreerd_in_inventaris</v>
       </c>
       <c r="D47" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E47" t="str">
-        <v>BER_ON</v>
+        <v>REGATT</v>
       </c>
       <c r="F47" t="str">
-        <v>Beroep onontvankelijk verklaard</v>
+        <v>Registratieattest</v>
       </c>
       <c r="G47" t="str">
         <v>null</v>
@@ -3174,22 +3174,22 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_onontvankelijk_verklaard_begeleidende_brief</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/registratieattest_begeleidende_brief</v>
       </c>
       <c r="B48" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C48" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_onontvankelijk_verklaard</v>
+        <v>null</v>
       </c>
       <c r="D48" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E48" t="str">
-        <v>BER_ON_BEG_BRIEF</v>
+        <v>REGATT_BEG_BRIEF</v>
       </c>
       <c r="F48" t="str">
-        <v>Begeleidende brief bij beroep onontvankelijk verklaard</v>
+        <v>Begeleidende brief bij een registratieattest</v>
       </c>
       <c r="G48" t="str">
         <v>null</v>
@@ -3233,22 +3233,22 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_verworpen</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/retour_afzender_procedurestuk</v>
       </c>
       <c r="B49" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C49" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/beroep_tegen_registratie_verworpen</v>
+        <v>null</v>
       </c>
       <c r="D49" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E49" t="str">
-        <v>BER_VERWN</v>
+        <v>RETOUR_AFZENDER_PROCEDURESTUK</v>
       </c>
       <c r="F49" t="str">
-        <v>Beroep verworpen</v>
+        <v>Retour afzender</v>
       </c>
       <c r="G49" t="str">
         <v>null</v>
@@ -3260,13 +3260,13 @@
         <v>null</v>
       </c>
       <c r="J49" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/procedurestuk</v>
       </c>
       <c r="K49" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/procedurestuk</v>
       </c>
       <c r="L49" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/procedurestuk</v>
       </c>
       <c r="M49" t="str">
         <v>null</v>
@@ -3292,25 +3292,25 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_verworpen_begeleidende_brief</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/stavingsstuk</v>
       </c>
       <c r="B50" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C50" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_verworpen</v>
+        <v>null</v>
       </c>
       <c r="D50" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E50" t="str">
-        <v>BER_VERWN_BEG_BRIEF</v>
+        <v>stavingsstuk</v>
       </c>
       <c r="F50" t="str">
-        <v>Begeleidende brief bij beroep verworpen</v>
+        <v>Stavingsstuk bij een vaststelling</v>
       </c>
       <c r="G50" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="H50" t="str">
         <v>null</v>
@@ -3319,19 +3319,19 @@
         <v>null</v>
       </c>
       <c r="J50" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
+        <v>null</v>
       </c>
       <c r="K50" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
+        <v>null</v>
       </c>
       <c r="L50" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/foto|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/varia|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/verslag</v>
       </c>
       <c r="M50" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/foto|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/varia|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/verslag</v>
       </c>
       <c r="N50" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/foto|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/varia|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/verslag</v>
       </c>
       <c r="O50" t="str">
         <v>null</v>
@@ -3351,7 +3351,7 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/varia</v>
       </c>
       <c r="B51" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -3363,13 +3363,13 @@
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E51" t="str">
-        <v>beslissingsstuk</v>
+        <v>VARIA</v>
       </c>
       <c r="F51" t="str">
-        <v>Stuk dat voortkomt uit een beslissing</v>
+        <v>Varia</v>
       </c>
       <c r="G51" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
+        <v>null</v>
       </c>
       <c r="H51" t="str">
         <v>null</v>
@@ -3378,19 +3378,19 @@
         <v>null</v>
       </c>
       <c r="J51" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/stavingsstuk</v>
       </c>
       <c r="K51" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/stavingsstuk</v>
       </c>
       <c r="L51" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_niet_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_niet_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_niet_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_niet_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_ingewilligd|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_ingewilligd_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_onontvankelijk_verklaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_onontvankelijk_verklaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_verworpen|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_verworpen_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/registratieattest|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/registratieattest_begeleidende_brief</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/stavingsstuk</v>
       </c>
       <c r="M51" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_niet_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_niet_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_niet_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_niet_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_ingewilligd|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_ingewilligd_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_onontvankelijk_verklaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_onontvankelijk_verklaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_verworpen|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_verworpen_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/registratieattest|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/registratieattest_begeleidende_brief</v>
+        <v>null</v>
       </c>
       <c r="N51" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_niet_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_niet_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_niet_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_niet_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_ingewilligd|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_ingewilligd_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_onontvankelijk_verklaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_onontvankelijk_verklaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_verworpen|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_verworpen_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/registratieattest|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/registratieattest_begeleidende_brief</v>
+        <v>null</v>
       </c>
       <c r="O51" t="str">
         <v>null</v>
@@ -3410,7 +3410,7 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/foto</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/verslag</v>
       </c>
       <c r="B52" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -3422,10 +3422,10 @@
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E52" t="str">
-        <v>FOTO</v>
+        <v>VERSLAG</v>
       </c>
       <c r="F52" t="str">
-        <v>Foto</v>
+        <v>Verslag</v>
       </c>
       <c r="G52" t="str">
         <v>null</v>
@@ -3469,7 +3469,7 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/inkomend_procedurestuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/buitenmuren</v>
       </c>
       <c r="B53" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -3478,13 +3478,13 @@
         <v>null</v>
       </c>
       <c r="D53" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/uitgesproken_gebrek</v>
       </c>
       <c r="E53" t="str">
-        <v>INKOMEND_PROCEDURESTUK</v>
+        <v>buitenmuren</v>
       </c>
       <c r="F53" t="str">
-        <v>Inkomend procedurestuk</v>
+        <v>Gebrek aan de toestand van buitenmuren</v>
       </c>
       <c r="G53" t="str">
         <v>null</v>
@@ -3496,13 +3496,13 @@
         <v>null</v>
       </c>
       <c r="J53" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/procedurestuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
       </c>
       <c r="K53" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/procedurestuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
       </c>
       <c r="L53" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/procedurestuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
       </c>
       <c r="M53" t="str">
         <v>null</v>
@@ -3511,13 +3511,13 @@
         <v>null</v>
       </c>
       <c r="O53" t="str">
-        <v>null</v>
+        <v>Buitenmuren</v>
       </c>
       <c r="P53" t="str">
-        <v>null</v>
+        <v>http://www.eionet.europa.eu/gemet/theme/5</v>
       </c>
       <c r="Q53" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/ns/verwaarlozing#vertoont_gebrek_ivm_buitenmuren</v>
       </c>
       <c r="R53" t="str">
         <v>null</v>
@@ -3528,7 +3528,7 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/procedurestuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/buitentimmerwerk</v>
       </c>
       <c r="B54" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -3537,16 +3537,16 @@
         <v>null</v>
       </c>
       <c r="D54" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/uitgesproken_gebrek</v>
       </c>
       <c r="E54" t="str">
-        <v>procedurestuk</v>
+        <v>buitentimmerwerk</v>
       </c>
       <c r="F54" t="str">
-        <v>Stuk gerelateerd aan een procedure</v>
+        <v>Gebrek aan de toestand van het buitentimmerwerk</v>
       </c>
       <c r="G54" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
+        <v>null</v>
       </c>
       <c r="H54" t="str">
         <v>null</v>
@@ -3555,28 +3555,28 @@
         <v>null</v>
       </c>
       <c r="J54" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
       </c>
       <c r="K54" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
       </c>
       <c r="L54" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/inkomend_procedurestuk|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/retour_afzender_procedurestuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
       </c>
       <c r="M54" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/inkomend_procedurestuk|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/retour_afzender_procedurestuk</v>
+        <v>null</v>
       </c>
       <c r="N54" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/inkomend_procedurestuk|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/retour_afzender_procedurestuk</v>
+        <v>null</v>
       </c>
       <c r="O54" t="str">
-        <v>null</v>
+        <v>Buitentimmerwerk</v>
       </c>
       <c r="P54" t="str">
-        <v>null</v>
+        <v>http://www.eionet.europa.eu/gemet/theme/5</v>
       </c>
       <c r="Q54" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/ns/verwaarlozing#vertoont_gebrek_ivm_buitentimmerwerk</v>
       </c>
       <c r="R54" t="str">
         <v>null</v>
@@ -3587,22 +3587,22 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/registratieattest</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakbedekking</v>
       </c>
       <c r="B55" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C55" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/geregistreerd_in_inventaris</v>
+        <v>null</v>
       </c>
       <c r="D55" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/uitgesproken_gebrek</v>
       </c>
       <c r="E55" t="str">
-        <v>REGATT</v>
+        <v>dakbedekking</v>
       </c>
       <c r="F55" t="str">
-        <v>Registratieattest</v>
+        <v>Gebrek aan de toestand van de dakbedekking</v>
       </c>
       <c r="G55" t="str">
         <v>null</v>
@@ -3614,13 +3614,13 @@
         <v>null</v>
       </c>
       <c r="J55" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
       </c>
       <c r="K55" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
       </c>
       <c r="L55" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
       </c>
       <c r="M55" t="str">
         <v>null</v>
@@ -3629,13 +3629,13 @@
         <v>null</v>
       </c>
       <c r="O55" t="str">
-        <v>null</v>
+        <v>Dakbedekking</v>
       </c>
       <c r="P55" t="str">
-        <v>null</v>
+        <v>http://www.eionet.europa.eu/gemet/theme/5</v>
       </c>
       <c r="Q55" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/ns/verwaarlozing#vertoont_gebrek_ivm_dakbedekking</v>
       </c>
       <c r="R55" t="str">
         <v>null</v>
@@ -3646,7 +3646,7 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/registratieattest_begeleidende_brief</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakgebinte</v>
       </c>
       <c r="B56" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -3655,13 +3655,13 @@
         <v>null</v>
       </c>
       <c r="D56" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/uitgesproken_gebrek</v>
       </c>
       <c r="E56" t="str">
-        <v>REGATT_BEG_BRIEF</v>
+        <v>dakgebinte</v>
       </c>
       <c r="F56" t="str">
-        <v>Begeleidende brief bij een registratieattest</v>
+        <v>Gebrek aan de toestand van het dakgebinte</v>
       </c>
       <c r="G56" t="str">
         <v>null</v>
@@ -3673,13 +3673,13 @@
         <v>null</v>
       </c>
       <c r="J56" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
       </c>
       <c r="K56" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
       </c>
       <c r="L56" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
       </c>
       <c r="M56" t="str">
         <v>null</v>
@@ -3688,13 +3688,13 @@
         <v>null</v>
       </c>
       <c r="O56" t="str">
-        <v>null</v>
+        <v>Dakgebinte</v>
       </c>
       <c r="P56" t="str">
-        <v>null</v>
+        <v>http://www.eionet.europa.eu/gemet/theme/5</v>
       </c>
       <c r="Q56" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/ns/verwaarlozing#vertoont_gebrek_ivm_dakgebinte</v>
       </c>
       <c r="R56" t="str">
         <v>null</v>
@@ -3705,7 +3705,7 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/retour_afzender_procedurestuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakgoten</v>
       </c>
       <c r="B57" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -3714,13 +3714,13 @@
         <v>null</v>
       </c>
       <c r="D57" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/uitgesproken_gebrek</v>
       </c>
       <c r="E57" t="str">
-        <v>RETOUR_AFZENDER_PROCEDURESTUK</v>
+        <v>dakgoten</v>
       </c>
       <c r="F57" t="str">
-        <v>Retour afzender</v>
+        <v>Gebrek aan de toestand van de dakgoten</v>
       </c>
       <c r="G57" t="str">
         <v>null</v>
@@ -3732,13 +3732,13 @@
         <v>null</v>
       </c>
       <c r="J57" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/procedurestuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
       </c>
       <c r="K57" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/procedurestuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
       </c>
       <c r="L57" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/procedurestuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
       </c>
       <c r="M57" t="str">
         <v>null</v>
@@ -3747,13 +3747,13 @@
         <v>null</v>
       </c>
       <c r="O57" t="str">
-        <v>null</v>
+        <v>Dakgoten</v>
       </c>
       <c r="P57" t="str">
-        <v>null</v>
+        <v>http://www.eionet.europa.eu/gemet/theme/5</v>
       </c>
       <c r="Q57" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/ns/verwaarlozing#vertoont_gebrek_ivm_dakgoten</v>
       </c>
       <c r="R57" t="str">
         <v>null</v>
@@ -3764,7 +3764,7 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/stavingsstuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
       </c>
       <c r="B58" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -3773,16 +3773,16 @@
         <v>null</v>
       </c>
       <c r="D58" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/uitgesproken_gebrek</v>
       </c>
       <c r="E58" t="str">
-        <v>stavingsstuk</v>
+        <v>gebouwonderdeel</v>
       </c>
       <c r="F58" t="str">
-        <v>Stavingsstuk bij een vaststelling</v>
+        <v>Gebrek aan de toestand van een gebouwonderdeel</v>
       </c>
       <c r="G58" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/uitgesproken_gebrek</v>
       </c>
       <c r="H58" t="str">
         <v>null</v>
@@ -3797,22 +3797,22 @@
         <v>null</v>
       </c>
       <c r="L58" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/foto|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/varia|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/verslag</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/buitenmuren|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/buitentimmerwerk|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakbedekking|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakgebinte|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakgoten|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/kroonlijst|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/liften|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/schoorstenen|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/trappen</v>
       </c>
       <c r="M58" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/foto|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/varia|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/verslag</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/buitenmuren|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/buitentimmerwerk|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakbedekking|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakgebinte|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakgoten|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/kroonlijst|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/liften|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/schoorstenen|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/trappen</v>
       </c>
       <c r="N58" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/foto|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/varia|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/verslag</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/buitenmuren|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/buitentimmerwerk|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakbedekking|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakgebinte|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakgoten|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/kroonlijst|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/liften|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/schoorstenen|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/trappen</v>
       </c>
       <c r="O58" t="str">
-        <v>null</v>
+        <v>Gebrek aan de toestand van een gebouwonderdeel</v>
       </c>
       <c r="P58" t="str">
-        <v>null</v>
+        <v>http://www.eionet.europa.eu/gemet/theme/5</v>
       </c>
       <c r="Q58" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/ns/verwaarlozing#vertoont_gebrek_ivm_gebouwonderdeel</v>
       </c>
       <c r="R58" t="str">
         <v>null</v>
@@ -3823,7 +3823,7 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/varia</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/kroonlijst</v>
       </c>
       <c r="B59" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -3832,13 +3832,13 @@
         <v>null</v>
       </c>
       <c r="D59" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/uitgesproken_gebrek</v>
       </c>
       <c r="E59" t="str">
-        <v>VARIA</v>
+        <v>kroonlijst</v>
       </c>
       <c r="F59" t="str">
-        <v>Varia</v>
+        <v>Gebrek aan de toestand van de kroonlijst</v>
       </c>
       <c r="G59" t="str">
         <v>null</v>
@@ -3850,13 +3850,13 @@
         <v>null</v>
       </c>
       <c r="J59" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/stavingsstuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
       </c>
       <c r="K59" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/stavingsstuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
       </c>
       <c r="L59" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/stavingsstuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
       </c>
       <c r="M59" t="str">
         <v>null</v>
@@ -3865,13 +3865,13 @@
         <v>null</v>
       </c>
       <c r="O59" t="str">
-        <v>null</v>
+        <v>Kroonlijst</v>
       </c>
       <c r="P59" t="str">
-        <v>null</v>
+        <v>http://www.eionet.europa.eu/gemet/theme/5</v>
       </c>
       <c r="Q59" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/ns/verwaarlozing#vertoont_gebrek_ivm_kroonlijst</v>
       </c>
       <c r="R59" t="str">
         <v>null</v>
@@ -3882,7 +3882,7 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/verslag</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/liften</v>
       </c>
       <c r="B60" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -3891,13 +3891,13 @@
         <v>null</v>
       </c>
       <c r="D60" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/uitgesproken_gebrek</v>
       </c>
       <c r="E60" t="str">
-        <v>VERSLAG</v>
+        <v>liften</v>
       </c>
       <c r="F60" t="str">
-        <v>Verslag</v>
+        <v>Gebrek aan de toestand van de liften</v>
       </c>
       <c r="G60" t="str">
         <v>null</v>
@@ -3909,13 +3909,13 @@
         <v>null</v>
       </c>
       <c r="J60" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/stavingsstuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
       </c>
       <c r="K60" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/stavingsstuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
       </c>
       <c r="L60" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/stavingsstuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
       </c>
       <c r="M60" t="str">
         <v>null</v>
@@ -3924,13 +3924,13 @@
         <v>null</v>
       </c>
       <c r="O60" t="str">
-        <v>null</v>
+        <v>Liften</v>
       </c>
       <c r="P60" t="str">
-        <v>null</v>
+        <v>http://www.eionet.europa.eu/gemet/theme/5</v>
       </c>
       <c r="Q60" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/ns/verwaarlozing#vertoont_gebrek_ivm_liften</v>
       </c>
       <c r="R60" t="str">
         <v>null</v>
@@ -3941,7 +3941,7 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/buitenmuren</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/reden_van_verwijderen_uit_inventaris:benutting_meer_dan_vijftig_percent</v>
       </c>
       <c r="B61" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -3950,16 +3950,16 @@
         <v>null</v>
       </c>
       <c r="D61" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/uitgesproken_gebrek</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/reden_van_verwijderen_uit_inventaris</v>
       </c>
       <c r="E61" t="str">
-        <v>buitenmuren</v>
+        <v>+50%</v>
       </c>
       <c r="F61" t="str">
-        <v>Gebrek aan de toestand van buitenmuren</v>
+        <v>Benutting van meer dan 50% conform de vergunde bestemming van het gebouw</v>
       </c>
       <c r="G61" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/reden_van_verwijderen_uit_inventaris</v>
       </c>
       <c r="H61" t="str">
         <v>null</v>
@@ -3968,13 +3968,13 @@
         <v>null</v>
       </c>
       <c r="J61" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
+        <v>null</v>
       </c>
       <c r="K61" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
+        <v>null</v>
       </c>
       <c r="L61" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
+        <v>null</v>
       </c>
       <c r="M61" t="str">
         <v>null</v>
@@ -3983,13 +3983,13 @@
         <v>null</v>
       </c>
       <c r="O61" t="str">
-        <v>Buitenmuren</v>
+        <v>null</v>
       </c>
       <c r="P61" t="str">
-        <v>http://www.eionet.europa.eu/gemet/theme/5</v>
+        <v>null</v>
       </c>
       <c r="Q61" t="str">
-        <v>https://data.omgeving.vlaanderen.be/ns/verwaarlozing#vertoont_gebrek_ivm_buitenmuren</v>
+        <v>null</v>
       </c>
       <c r="R61" t="str">
         <v>null</v>
@@ -4000,7 +4000,7 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/buitentimmerwerk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/reden_van_verwijderen_uit_inventaris:functiewijziging</v>
       </c>
       <c r="B62" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -4009,16 +4009,16 @@
         <v>null</v>
       </c>
       <c r="D62" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/uitgesproken_gebrek</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/reden_van_verwijderen_uit_inventaris</v>
       </c>
       <c r="E62" t="str">
-        <v>buitentimmerwerk</v>
+        <v>functiewijziging</v>
       </c>
       <c r="F62" t="str">
-        <v>Gebrek aan de toestand van het buitentimmerwerk</v>
+        <v>Functiewijziging doorgevoerd</v>
       </c>
       <c r="G62" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/reden_van_verwijderen_uit_inventaris</v>
       </c>
       <c r="H62" t="str">
         <v>null</v>
@@ -4027,13 +4027,13 @@
         <v>null</v>
       </c>
       <c r="J62" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
+        <v>null</v>
       </c>
       <c r="K62" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
+        <v>null</v>
       </c>
       <c r="L62" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
+        <v>null</v>
       </c>
       <c r="M62" t="str">
         <v>null</v>
@@ -4042,13 +4042,13 @@
         <v>null</v>
       </c>
       <c r="O62" t="str">
-        <v>Buitentimmerwerk</v>
+        <v>null</v>
       </c>
       <c r="P62" t="str">
-        <v>http://www.eionet.europa.eu/gemet/theme/5</v>
+        <v>null</v>
       </c>
       <c r="Q62" t="str">
-        <v>https://data.omgeving.vlaanderen.be/ns/verwaarlozing#vertoont_gebrek_ivm_buitentimmerwerk</v>
+        <v>null</v>
       </c>
       <c r="R62" t="str">
         <v>null</v>
@@ -4059,7 +4059,7 @@
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakbedekking</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/reden_van_verwijderen_uit_inventaris:gesloopt</v>
       </c>
       <c r="B63" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -4068,16 +4068,16 @@
         <v>null</v>
       </c>
       <c r="D63" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/uitgesproken_gebrek</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/reden_van_verwijderen_uit_inventaris</v>
       </c>
       <c r="E63" t="str">
-        <v>dakbedekking</v>
+        <v>gesloopt</v>
       </c>
       <c r="F63" t="str">
-        <v>Gebrek aan de toestand van de dakbedekking</v>
+        <v>De bedrijfsruimte is gesloopt</v>
       </c>
       <c r="G63" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/reden_van_verwijderen_uit_inventaris</v>
       </c>
       <c r="H63" t="str">
         <v>null</v>
@@ -4086,13 +4086,13 @@
         <v>null</v>
       </c>
       <c r="J63" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
+        <v>null</v>
       </c>
       <c r="K63" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
+        <v>null</v>
       </c>
       <c r="L63" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
+        <v>null</v>
       </c>
       <c r="M63" t="str">
         <v>null</v>
@@ -4101,13 +4101,13 @@
         <v>null</v>
       </c>
       <c r="O63" t="str">
-        <v>Dakbedekking</v>
+        <v>null</v>
       </c>
       <c r="P63" t="str">
-        <v>http://www.eionet.europa.eu/gemet/theme/5</v>
+        <v>null</v>
       </c>
       <c r="Q63" t="str">
-        <v>https://data.omgeving.vlaanderen.be/ns/verwaarlozing#vertoont_gebrek_ivm_dakbedekking</v>
+        <v>null</v>
       </c>
       <c r="R63" t="str">
         <v>null</v>
@@ -4118,7 +4118,7 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakgebinte</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/reden_van_verwijderen_uit_inventaris:heffing</v>
       </c>
       <c r="B64" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -4127,16 +4127,16 @@
         <v>null</v>
       </c>
       <c r="D64" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/uitgesproken_gebrek</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/reden_van_verwijderen_uit_inventaris</v>
       </c>
       <c r="E64" t="str">
-        <v>dakgebinte</v>
+        <v>heffing</v>
       </c>
       <c r="F64" t="str">
-        <v>Gebrek aan de toestand van het dakgebinte</v>
+        <v>Procedure heffing</v>
       </c>
       <c r="G64" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/reden_van_verwijderen_uit_inventaris</v>
       </c>
       <c r="H64" t="str">
         <v>null</v>
@@ -4145,13 +4145,13 @@
         <v>null</v>
       </c>
       <c r="J64" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
+        <v>null</v>
       </c>
       <c r="K64" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
+        <v>null</v>
       </c>
       <c r="L64" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
+        <v>null</v>
       </c>
       <c r="M64" t="str">
         <v>null</v>
@@ -4160,13 +4160,13 @@
         <v>null</v>
       </c>
       <c r="O64" t="str">
-        <v>Dakgebinte</v>
+        <v>null</v>
       </c>
       <c r="P64" t="str">
-        <v>http://www.eionet.europa.eu/gemet/theme/5</v>
+        <v>null</v>
       </c>
       <c r="Q64" t="str">
-        <v>https://data.omgeving.vlaanderen.be/ns/verwaarlozing#vertoont_gebrek_ivm_dakgebinte</v>
+        <v>null</v>
       </c>
       <c r="R64" t="str">
         <v>null</v>
@@ -4177,7 +4177,7 @@
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakgoten</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/reden_van_verwijderen_uit_inventaris:nieuwe_invulling</v>
       </c>
       <c r="B65" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -4186,16 +4186,16 @@
         <v>null</v>
       </c>
       <c r="D65" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/uitgesproken_gebrek</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/reden_van_verwijderen_uit_inventaris</v>
       </c>
       <c r="E65" t="str">
-        <v>dakgoten</v>
+        <v>nieuwe_invulling</v>
       </c>
       <c r="F65" t="str">
-        <v>Gebrek aan de toestand van de dakgoten</v>
+        <v>Nieuwe invulling gegeven conform de vergunde bestemming</v>
       </c>
       <c r="G65" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/reden_van_verwijderen_uit_inventaris</v>
       </c>
       <c r="H65" t="str">
         <v>null</v>
@@ -4204,13 +4204,13 @@
         <v>null</v>
       </c>
       <c r="J65" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
+        <v>null</v>
       </c>
       <c r="K65" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
+        <v>null</v>
       </c>
       <c r="L65" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
+        <v>null</v>
       </c>
       <c r="M65" t="str">
         <v>null</v>
@@ -4219,13 +4219,13 @@
         <v>null</v>
       </c>
       <c r="O65" t="str">
-        <v>Dakgoten</v>
+        <v>null</v>
       </c>
       <c r="P65" t="str">
-        <v>http://www.eionet.europa.eu/gemet/theme/5</v>
+        <v>null</v>
       </c>
       <c r="Q65" t="str">
-        <v>https://data.omgeving.vlaanderen.be/ns/verwaarlozing#vertoont_gebrek_ivm_dakgoten</v>
+        <v>null</v>
       </c>
       <c r="R65" t="str">
         <v>null</v>
@@ -4236,7 +4236,7 @@
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/reden_van_verwijderen_uit_inventaris:onteigening</v>
       </c>
       <c r="B66" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -4245,16 +4245,16 @@
         <v>null</v>
       </c>
       <c r="D66" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/uitgesproken_gebrek</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/reden_van_verwijderen_uit_inventaris</v>
       </c>
       <c r="E66" t="str">
-        <v>gebouwonderdeel</v>
+        <v>onteigening</v>
       </c>
       <c r="F66" t="str">
-        <v>Gebrek aan de toestand van een gebouwonderdeel</v>
+        <v>Er is een onteigening</v>
       </c>
       <c r="G66" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/uitgesproken_gebrek</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/reden_van_verwijderen_uit_inventaris</v>
       </c>
       <c r="H66" t="str">
         <v>null</v>
@@ -4269,22 +4269,22 @@
         <v>null</v>
       </c>
       <c r="L66" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/buitenmuren|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/buitentimmerwerk|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakbedekking|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakgebinte|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakgoten|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/kroonlijst|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/liften|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/schoorstenen|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/trappen</v>
+        <v>null</v>
       </c>
       <c r="M66" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/buitenmuren|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/buitentimmerwerk|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakbedekking|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakgebinte|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakgoten|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/kroonlijst|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/liften|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/schoorstenen|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/trappen</v>
+        <v>null</v>
       </c>
       <c r="N66" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/buitenmuren|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/buitentimmerwerk|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakbedekking|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakgebinte|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakgoten|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/kroonlijst|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/liften|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/schoorstenen|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/trappen</v>
+        <v>null</v>
       </c>
       <c r="O66" t="str">
-        <v>Gebrek aan de toestand van een gebouwonderdeel</v>
+        <v>null</v>
       </c>
       <c r="P66" t="str">
-        <v>http://www.eionet.europa.eu/gemet/theme/5</v>
+        <v>null</v>
       </c>
       <c r="Q66" t="str">
-        <v>https://data.omgeving.vlaanderen.be/ns/verwaarlozing#vertoont_gebrek_ivm_gebouwonderdeel</v>
+        <v>null</v>
       </c>
       <c r="R66" t="str">
         <v>null</v>
@@ -4295,7 +4295,7 @@
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/kroonlijst</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/reden_van_verwijderen_uit_inventaris:opgeheven</v>
       </c>
       <c r="B67" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -4304,16 +4304,16 @@
         <v>null</v>
       </c>
       <c r="D67" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/uitgesproken_gebrek</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/reden_van_verwijderen_uit_inventaris</v>
       </c>
       <c r="E67" t="str">
-        <v>kroonlijst</v>
+        <v>opgeheven</v>
       </c>
       <c r="F67" t="str">
-        <v>Gebrek aan de toestand van de kroonlijst</v>
+        <v>Verwaarlozing is opgeheven</v>
       </c>
       <c r="G67" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/reden_van_verwijderen_uit_inventaris</v>
       </c>
       <c r="H67" t="str">
         <v>null</v>
@@ -4322,13 +4322,13 @@
         <v>null</v>
       </c>
       <c r="J67" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
+        <v>null</v>
       </c>
       <c r="K67" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
+        <v>null</v>
       </c>
       <c r="L67" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
+        <v>null</v>
       </c>
       <c r="M67" t="str">
         <v>null</v>
@@ -4337,13 +4337,13 @@
         <v>null</v>
       </c>
       <c r="O67" t="str">
-        <v>Kroonlijst</v>
+        <v>null</v>
       </c>
       <c r="P67" t="str">
-        <v>http://www.eionet.europa.eu/gemet/theme/5</v>
+        <v>null</v>
       </c>
       <c r="Q67" t="str">
-        <v>https://data.omgeving.vlaanderen.be/ns/verwaarlozing#vertoont_gebrek_ivm_kroonlijst</v>
+        <v>null</v>
       </c>
       <c r="R67" t="str">
         <v>null</v>
@@ -4354,7 +4354,7 @@
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/liften</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/reden_van_verwijderen_uit_inventaris:rechtbank</v>
       </c>
       <c r="B68" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -4363,16 +4363,16 @@
         <v>null</v>
       </c>
       <c r="D68" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/uitgesproken_gebrek</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/reden_van_verwijderen_uit_inventaris</v>
       </c>
       <c r="E68" t="str">
-        <v>liften</v>
+        <v>rechtbank</v>
       </c>
       <c r="F68" t="str">
-        <v>Gebrek aan de toestand van de liften</v>
+        <v>Procedure rechtbank</v>
       </c>
       <c r="G68" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/reden_van_verwijderen_uit_inventaris</v>
       </c>
       <c r="H68" t="str">
         <v>null</v>
@@ -4381,13 +4381,13 @@
         <v>null</v>
       </c>
       <c r="J68" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
+        <v>null</v>
       </c>
       <c r="K68" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
+        <v>null</v>
       </c>
       <c r="L68" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
+        <v>null</v>
       </c>
       <c r="M68" t="str">
         <v>null</v>
@@ -4396,13 +4396,13 @@
         <v>null</v>
       </c>
       <c r="O68" t="str">
-        <v>Liften</v>
+        <v>null</v>
       </c>
       <c r="P68" t="str">
-        <v>http://www.eionet.europa.eu/gemet/theme/5</v>
+        <v>null</v>
       </c>
       <c r="Q68" t="str">
-        <v>https://data.omgeving.vlaanderen.be/ns/verwaarlozing#vertoont_gebrek_ivm_liften</v>
+        <v>null</v>
       </c>
       <c r="R68" t="str">
         <v>null</v>
@@ -4885,7 +4885,7 @@
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/rol</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/reden_van_verwijderen_uit_inventaris</v>
       </c>
       <c r="B77" t="str">
         <v>http://www.w3.org/2004/02/skos/core#ConceptScheme</v>
@@ -4897,19 +4897,19 @@
         <v>null</v>
       </c>
       <c r="E77" t="str">
-        <v>cs_rol</v>
+        <v>cs_reden_van_verwijderen_uit_inventaris</v>
       </c>
       <c r="F77" t="str">
-        <v>Conceptschema over rollen van agenten binnen procedures in het kader van leegstaande en verwaarloosde bedrijfsruimten.</v>
+        <v>Conceptschema over redenen van verwijderen uit inventaris in het kader van leegstaande en verwaarloosde bedrijfsruimten.</v>
       </c>
       <c r="G77" t="str">
         <v>null</v>
       </c>
       <c r="H77" t="str">
-        <v>Conceptschema over rollen van agenten binnen procedures in het kader van leegstaande en verwaarloosde bedrijfsruimten.</v>
+        <v>Redenen van verwijderen uit inventaris</v>
       </c>
       <c r="I77" t="str">
-        <v>Conceptschema over rollen van agenten binnen procedures in het kader van leegstaande en verwaarloosde bedrijfsruimten.</v>
+        <v>Redenen van verwijderen uit inventaris</v>
       </c>
       <c r="J77" t="str">
         <v>null</v>
@@ -4939,12 +4939,12 @@
         <v>https://data.omgeving.vlaanderen.be/id/dataset/codelijst-verwaarlozing</v>
       </c>
       <c r="S77" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/rol/bewindvoerder|https://data.omgeving.vlaanderen.be/id/concept/leegstand/rol/curator|https://data.omgeving.vlaanderen.be/id/concept/leegstand/rol/eigenaar|https://data.omgeving.vlaanderen.be/id/concept/leegstand/rol/instrumenterend_ambtenaar|https://data.omgeving.vlaanderen.be/id/concept/leegstand/rol/raadsman</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/reden_van_verwijderen_uit_inventaris:benutting_meer_dan_vijftig_percent|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/reden_van_verwijderen_uit_inventaris:functiewijziging|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/reden_van_verwijderen_uit_inventaris:gesloopt|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/reden_van_verwijderen_uit_inventaris:heffing|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/reden_van_verwijderen_uit_inventaris:nieuwe_invulling|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/reden_van_verwijderen_uit_inventaris:onteigening|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/reden_van_verwijderen_uit_inventaris:opgeheven|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/reden_van_verwijderen_uit_inventaris:rechtbank</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/schrapping</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/rol</v>
       </c>
       <c r="B78" t="str">
         <v>http://www.w3.org/2004/02/skos/core#ConceptScheme</v>
@@ -4956,19 +4956,19 @@
         <v>null</v>
       </c>
       <c r="E78" t="str">
-        <v>cs_schrapping</v>
+        <v>cs_rol</v>
       </c>
       <c r="F78" t="str">
-        <v>Conceptschema over redenen van schapping in het kader van leegstaande en verwaarloosde bedrijfsruimten.</v>
+        <v>Conceptschema over rollen van agenten binnen procedures in het kader van leegstaande en verwaarloosde bedrijfsruimten.</v>
       </c>
       <c r="G78" t="str">
         <v>null</v>
       </c>
       <c r="H78" t="str">
-        <v>Redenen van schrapping</v>
+        <v>Conceptschema over rollen van agenten binnen procedures in het kader van leegstaande en verwaarloosde bedrijfsruimten.</v>
       </c>
       <c r="I78" t="str">
-        <v>Redenen van schrapping</v>
+        <v>Conceptschema over rollen van agenten binnen procedures in het kader van leegstaande en verwaarloosde bedrijfsruimten.</v>
       </c>
       <c r="J78" t="str">
         <v>null</v>
@@ -4998,7 +4998,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/dataset/codelijst-verwaarlozing</v>
       </c>
       <c r="S78" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/schrapping/benutting_meer_dan_vijftig_percent|https://data.omgeving.vlaanderen.be/id/concept/leegstand/schrapping/functiewijziging|https://data.omgeving.vlaanderen.be/id/concept/leegstand/schrapping/gesloopt|https://data.omgeving.vlaanderen.be/id/concept/leegstand/schrapping/heffing|https://data.omgeving.vlaanderen.be/id/concept/leegstand/schrapping/nieuwe_invulling|https://data.omgeving.vlaanderen.be/id/concept/leegstand/schrapping/onteigening|https://data.omgeving.vlaanderen.be/id/concept/leegstand/schrapping/opgeheven|https://data.omgeving.vlaanderen.be/id/concept/leegstand/schrapping/rechtbank</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/rol/bewindvoerder|https://data.omgeving.vlaanderen.be/id/concept/leegstand/rol/curator|https://data.omgeving.vlaanderen.be/id/concept/leegstand/rol/eigenaar|https://data.omgeving.vlaanderen.be/id/concept/leegstand/rol/instrumenterend_ambtenaar|https://data.omgeving.vlaanderen.be/id/concept/leegstand/rol/raadsman</v>
       </c>
     </row>
     <row r="79">

</xml_diff>

<commit_message>
LVBR-386: Fix na vergeten config aanpassing
</commit_message>
<xml_diff>
--- a/src/main/resources/be/vlaanderen/omgeving/data/id/conceptscheme/verwaarlozing/verwaarlozing.xlsx
+++ b/src/main/resources/be/vlaanderen/omgeving/data/id/conceptscheme/verwaarlozing/verwaarlozing.xlsx
@@ -1758,7 +1758,7 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/rol/bewindvoerder</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/reden_van_verwijderen_uit_inventaris/benutting_meer_dan_vijftig_percent</v>
       </c>
       <c r="B24" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -1767,16 +1767,16 @@
         <v>null</v>
       </c>
       <c r="D24" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/rol</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/reden_van_verwijderen_uit_inventaris</v>
       </c>
       <c r="E24" t="str">
-        <v>null</v>
+        <v>+50%</v>
       </c>
       <c r="F24" t="str">
-        <v>Bewindvoerder</v>
+        <v>Benutting van meer dan 50% conform de vergunde bestemming van het gebouw</v>
       </c>
       <c r="G24" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/rol</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/reden_van_verwijderen_uit_inventaris</v>
       </c>
       <c r="H24" t="str">
         <v>null</v>
@@ -1817,7 +1817,7 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/rol/curator</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/reden_van_verwijderen_uit_inventaris/functiewijziging</v>
       </c>
       <c r="B25" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -1826,16 +1826,16 @@
         <v>null</v>
       </c>
       <c r="D25" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/rol</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/reden_van_verwijderen_uit_inventaris</v>
       </c>
       <c r="E25" t="str">
-        <v>null</v>
+        <v>functiewijziging</v>
       </c>
       <c r="F25" t="str">
-        <v>Curator</v>
+        <v>Functiewijziging doorgevoerd</v>
       </c>
       <c r="G25" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/rol</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/reden_van_verwijderen_uit_inventaris</v>
       </c>
       <c r="H25" t="str">
         <v>null</v>
@@ -1876,7 +1876,7 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/rol/eigenaar</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/reden_van_verwijderen_uit_inventaris/gesloopt</v>
       </c>
       <c r="B26" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -1885,22 +1885,22 @@
         <v>null</v>
       </c>
       <c r="D26" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/rol</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/reden_van_verwijderen_uit_inventaris</v>
       </c>
       <c r="E26" t="str">
-        <v>null</v>
+        <v>gesloopt</v>
       </c>
       <c r="F26" t="str">
-        <v>Eigenaar</v>
+        <v>De bedrijfsruimte is gesloopt</v>
       </c>
       <c r="G26" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/rol</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/reden_van_verwijderen_uit_inventaris</v>
       </c>
       <c r="H26" t="str">
-        <v>De houder van een van de volgende zakelijke rechten met betrekking tot een bedrijfsgebouw: de volle eigendom, het recht van opstal of van erfpacht, het vruchtgebruik</v>
+        <v>null</v>
       </c>
       <c r="I26" t="str">
-        <v>De houder van een van de volgende zakelijke rechten met betrekking tot een bedrijfsgebouw: de volle eigendom, het recht van opstal of van erfpacht, het vruchtgebruik</v>
+        <v>null</v>
       </c>
       <c r="J26" t="str">
         <v>null</v>
@@ -1935,7 +1935,7 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/rol/instrumenterend_ambtenaar</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/reden_van_verwijderen_uit_inventaris/heffing</v>
       </c>
       <c r="B27" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -1944,22 +1944,22 @@
         <v>null</v>
       </c>
       <c r="D27" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/rol</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/reden_van_verwijderen_uit_inventaris</v>
       </c>
       <c r="E27" t="str">
-        <v>null</v>
+        <v>heffing</v>
       </c>
       <c r="F27" t="str">
-        <v>Instrumenterend ambtenaar</v>
+        <v>Procedure heffing</v>
       </c>
       <c r="G27" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/rol</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/reden_van_verwijderen_uit_inventaris</v>
       </c>
       <c r="H27" t="str">
-        <v>Iedere persoon of instelling die ertoe gemachtigd is aktes van eigendomsoverdracht te verlijden</v>
+        <v>null</v>
       </c>
       <c r="I27" t="str">
-        <v>Iedere persoon of instelling die ertoe gemachtigd is aktes van eigendomsoverdracht te verlijden</v>
+        <v>null</v>
       </c>
       <c r="J27" t="str">
         <v>null</v>
@@ -1994,7 +1994,7 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/rol/raadsman</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/reden_van_verwijderen_uit_inventaris/nieuwe_invulling</v>
       </c>
       <c r="B28" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -2003,16 +2003,16 @@
         <v>null</v>
       </c>
       <c r="D28" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/rol</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/reden_van_verwijderen_uit_inventaris</v>
       </c>
       <c r="E28" t="str">
-        <v>null</v>
+        <v>nieuwe_invulling</v>
       </c>
       <c r="F28" t="str">
-        <v>Raadsman</v>
+        <v>Nieuwe invulling gegeven conform de vergunde bestemming</v>
       </c>
       <c r="G28" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/rol</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/reden_van_verwijderen_uit_inventaris</v>
       </c>
       <c r="H28" t="str">
         <v>null</v>
@@ -2053,25 +2053,25 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_aanvaard</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/reden_van_verwijderen_uit_inventaris/onteigening</v>
       </c>
       <c r="B29" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C29" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/aanvraag_opschorting_heffing_aanvaard</v>
+        <v>null</v>
       </c>
       <c r="D29" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/reden_van_verwijderen_uit_inventaris</v>
       </c>
       <c r="E29" t="str">
-        <v>OPSCH_ANVRD</v>
+        <v>onteigening</v>
       </c>
       <c r="F29" t="str">
-        <v>Opschorting aanvaard</v>
+        <v>Er is een onteigening</v>
       </c>
       <c r="G29" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/reden_van_verwijderen_uit_inventaris</v>
       </c>
       <c r="H29" t="str">
         <v>null</v>
@@ -2080,13 +2080,13 @@
         <v>null</v>
       </c>
       <c r="J29" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
+        <v>null</v>
       </c>
       <c r="K29" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
+        <v>null</v>
       </c>
       <c r="L29" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
+        <v>null</v>
       </c>
       <c r="M29" t="str">
         <v>null</v>
@@ -2112,25 +2112,25 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_aanvaard_begeleidende_brief</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/reden_van_verwijderen_uit_inventaris/opgeheven</v>
       </c>
       <c r="B30" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C30" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_aanvaard</v>
+        <v>null</v>
       </c>
       <c r="D30" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/reden_van_verwijderen_uit_inventaris</v>
       </c>
       <c r="E30" t="str">
-        <v>OPSCH_ANVRD_BEG_BRIEF</v>
+        <v>opgeheven</v>
       </c>
       <c r="F30" t="str">
-        <v>Begeleidende brief bij opschorting aanvaard</v>
+        <v>Verwaarlozing is opgeheven</v>
       </c>
       <c r="G30" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/reden_van_verwijderen_uit_inventaris</v>
       </c>
       <c r="H30" t="str">
         <v>null</v>
@@ -2139,13 +2139,13 @@
         <v>null</v>
       </c>
       <c r="J30" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
+        <v>null</v>
       </c>
       <c r="K30" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
+        <v>null</v>
       </c>
       <c r="L30" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
+        <v>null</v>
       </c>
       <c r="M30" t="str">
         <v>null</v>
@@ -2171,25 +2171,25 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_niet_aanvaard</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/reden_van_verwijderen_uit_inventaris/rechtbank</v>
       </c>
       <c r="B31" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C31" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/aanvraag_opschorting_heffing_niet_aanvaard</v>
+        <v>null</v>
       </c>
       <c r="D31" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/reden_van_verwijderen_uit_inventaris</v>
       </c>
       <c r="E31" t="str">
-        <v>OPSCH_NANVRD</v>
+        <v>rechtbank</v>
       </c>
       <c r="F31" t="str">
-        <v>Opschorting niet aanvaard</v>
+        <v>Procedure rechtbank</v>
       </c>
       <c r="G31" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/reden_van_verwijderen_uit_inventaris</v>
       </c>
       <c r="H31" t="str">
         <v>null</v>
@@ -2198,13 +2198,13 @@
         <v>null</v>
       </c>
       <c r="J31" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
+        <v>null</v>
       </c>
       <c r="K31" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
+        <v>null</v>
       </c>
       <c r="L31" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
+        <v>null</v>
       </c>
       <c r="M31" t="str">
         <v>null</v>
@@ -2230,25 +2230,25 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_niet_aanvaard_begeleidende_brief</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/rol/bewindvoerder</v>
       </c>
       <c r="B32" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C32" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_niet_aanvaard</v>
+        <v>null</v>
       </c>
       <c r="D32" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/rol</v>
       </c>
       <c r="E32" t="str">
-        <v>OPSCH_NANVRD_BEG_BRIEF</v>
+        <v>null</v>
       </c>
       <c r="F32" t="str">
-        <v>Begeleidende brief bij opschorting niet aanvaard</v>
+        <v>Bewindvoerder</v>
       </c>
       <c r="G32" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/rol</v>
       </c>
       <c r="H32" t="str">
         <v>null</v>
@@ -2257,13 +2257,13 @@
         <v>null</v>
       </c>
       <c r="J32" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
+        <v>null</v>
       </c>
       <c r="K32" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
+        <v>null</v>
       </c>
       <c r="L32" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
+        <v>null</v>
       </c>
       <c r="M32" t="str">
         <v>null</v>
@@ -2289,25 +2289,25 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_aanvaard</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/rol/curator</v>
       </c>
       <c r="B33" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C33" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/aanvraag_schrapping_aanvaard</v>
+        <v>null</v>
       </c>
       <c r="D33" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/rol</v>
       </c>
       <c r="E33" t="str">
-        <v>SCHR_ANVRD</v>
+        <v>null</v>
       </c>
       <c r="F33" t="str">
-        <v>Schrapping aanvaard</v>
+        <v>Curator</v>
       </c>
       <c r="G33" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/rol</v>
       </c>
       <c r="H33" t="str">
         <v>null</v>
@@ -2316,13 +2316,13 @@
         <v>null</v>
       </c>
       <c r="J33" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
+        <v>null</v>
       </c>
       <c r="K33" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
+        <v>null</v>
       </c>
       <c r="L33" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
+        <v>null</v>
       </c>
       <c r="M33" t="str">
         <v>null</v>
@@ -2348,40 +2348,40 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_aanvaard_begeleidende_brief</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/rol/eigenaar</v>
       </c>
       <c r="B34" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C34" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_aanvaard</v>
+        <v>null</v>
       </c>
       <c r="D34" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/rol</v>
       </c>
       <c r="E34" t="str">
-        <v>SCHR_ANVRD_BEG_BRIEF</v>
+        <v>null</v>
       </c>
       <c r="F34" t="str">
-        <v>Begeleidende brief bij schrapping aanvaard</v>
+        <v>Eigenaar</v>
       </c>
       <c r="G34" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/rol</v>
       </c>
       <c r="H34" t="str">
-        <v>null</v>
+        <v>De houder van een van de volgende zakelijke rechten met betrekking tot een bedrijfsgebouw: de volle eigendom, het recht van opstal of van erfpacht, het vruchtgebruik</v>
       </c>
       <c r="I34" t="str">
-        <v>null</v>
+        <v>De houder van een van de volgende zakelijke rechten met betrekking tot een bedrijfsgebouw: de volle eigendom, het recht van opstal of van erfpacht, het vruchtgebruik</v>
       </c>
       <c r="J34" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
+        <v>null</v>
       </c>
       <c r="K34" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
+        <v>null</v>
       </c>
       <c r="L34" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
+        <v>null</v>
       </c>
       <c r="M34" t="str">
         <v>null</v>
@@ -2407,40 +2407,40 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_niet_aanvaard</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/rol/instrumenterend_ambtenaar</v>
       </c>
       <c r="B35" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C35" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/aanvraag_schrapping_niet_aanvaard</v>
+        <v>null</v>
       </c>
       <c r="D35" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/rol</v>
       </c>
       <c r="E35" t="str">
-        <v>SCHR_NANVRD</v>
+        <v>null</v>
       </c>
       <c r="F35" t="str">
-        <v>Schrapping niet aanvaard</v>
+        <v>Instrumenterend ambtenaar</v>
       </c>
       <c r="G35" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/rol</v>
       </c>
       <c r="H35" t="str">
-        <v>null</v>
+        <v>Iedere persoon of instelling die ertoe gemachtigd is aktes van eigendomsoverdracht te verlijden</v>
       </c>
       <c r="I35" t="str">
-        <v>null</v>
+        <v>Iedere persoon of instelling die ertoe gemachtigd is aktes van eigendomsoverdracht te verlijden</v>
       </c>
       <c r="J35" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
+        <v>null</v>
       </c>
       <c r="K35" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
+        <v>null</v>
       </c>
       <c r="L35" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
+        <v>null</v>
       </c>
       <c r="M35" t="str">
         <v>null</v>
@@ -2466,25 +2466,25 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_niet_aanvaard_begeleidende_brief</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/rol/raadsman</v>
       </c>
       <c r="B36" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C36" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_niet_aanvaard</v>
+        <v>null</v>
       </c>
       <c r="D36" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/rol</v>
       </c>
       <c r="E36" t="str">
-        <v>SCHR_NANVRD_BEG_BRIEF</v>
+        <v>null</v>
       </c>
       <c r="F36" t="str">
-        <v>Begeleidende brief bij schrapping niet aanvaard</v>
+        <v>Raadsman</v>
       </c>
       <c r="G36" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/rol</v>
       </c>
       <c r="H36" t="str">
         <v>null</v>
@@ -2493,13 +2493,13 @@
         <v>null</v>
       </c>
       <c r="J36" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
+        <v>null</v>
       </c>
       <c r="K36" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
+        <v>null</v>
       </c>
       <c r="L36" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
+        <v>null</v>
       </c>
       <c r="M36" t="str">
         <v>null</v>
@@ -2525,22 +2525,22 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_ingewilligd</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_aanvaard</v>
       </c>
       <c r="B37" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C37" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/beroep_tegen_registratie_ingewilligd</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/aanvraag_opschorting_heffing_aanvaard</v>
       </c>
       <c r="D37" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E37" t="str">
-        <v>BER_INGWD</v>
+        <v>OPSCH_ANVRD</v>
       </c>
       <c r="F37" t="str">
-        <v>Beroep ingewilligd</v>
+        <v>Opschorting aanvaard</v>
       </c>
       <c r="G37" t="str">
         <v>null</v>
@@ -2584,22 +2584,22 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_ingewilligd_begeleidende_brief</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_aanvaard_begeleidende_brief</v>
       </c>
       <c r="B38" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C38" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_ingewilligd</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_aanvaard</v>
       </c>
       <c r="D38" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E38" t="str">
-        <v>BER_INGWD_BEG_BRIEF</v>
+        <v>OPSCH_ANVRD_BEG_BRIEF</v>
       </c>
       <c r="F38" t="str">
-        <v>Begeleidende brief bij beroep ingewilligd</v>
+        <v>Begeleidende brief bij opschorting aanvaard</v>
       </c>
       <c r="G38" t="str">
         <v>null</v>
@@ -2643,22 +2643,22 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_onontvankelijk_verklaard</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_niet_aanvaard</v>
       </c>
       <c r="B39" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C39" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/beroep_tegen_registratie_onontvankelijk_verklaard</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/aanvraag_opschorting_heffing_niet_aanvaard</v>
       </c>
       <c r="D39" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E39" t="str">
-        <v>BER_ON</v>
+        <v>OPSCH_NANVRD</v>
       </c>
       <c r="F39" t="str">
-        <v>Beroep onontvankelijk verklaard</v>
+        <v>Opschorting niet aanvaard</v>
       </c>
       <c r="G39" t="str">
         <v>null</v>
@@ -2702,22 +2702,22 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_onontvankelijk_verklaard_begeleidende_brief</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_niet_aanvaard_begeleidende_brief</v>
       </c>
       <c r="B40" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C40" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_onontvankelijk_verklaard</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_niet_aanvaard</v>
       </c>
       <c r="D40" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E40" t="str">
-        <v>BER_ON_BEG_BRIEF</v>
+        <v>OPSCH_NANVRD_BEG_BRIEF</v>
       </c>
       <c r="F40" t="str">
-        <v>Begeleidende brief bij beroep onontvankelijk verklaard</v>
+        <v>Begeleidende brief bij opschorting niet aanvaard</v>
       </c>
       <c r="G40" t="str">
         <v>null</v>
@@ -2761,22 +2761,22 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_verworpen</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_aanvaard</v>
       </c>
       <c r="B41" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C41" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/beroep_tegen_registratie_verworpen</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/aanvraag_schrapping_aanvaard</v>
       </c>
       <c r="D41" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E41" t="str">
-        <v>BER_VERWN</v>
+        <v>SCHR_ANVRD</v>
       </c>
       <c r="F41" t="str">
-        <v>Beroep verworpen</v>
+        <v>Schrapping aanvaard</v>
       </c>
       <c r="G41" t="str">
         <v>null</v>
@@ -2820,22 +2820,22 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_verworpen_begeleidende_brief</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_aanvaard_begeleidende_brief</v>
       </c>
       <c r="B42" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C42" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_verworpen</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_aanvaard</v>
       </c>
       <c r="D42" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E42" t="str">
-        <v>BER_VERWN_BEG_BRIEF</v>
+        <v>SCHR_ANVRD_BEG_BRIEF</v>
       </c>
       <c r="F42" t="str">
-        <v>Begeleidende brief bij beroep verworpen</v>
+        <v>Begeleidende brief bij schrapping aanvaard</v>
       </c>
       <c r="G42" t="str">
         <v>null</v>
@@ -2879,25 +2879,25 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_niet_aanvaard</v>
       </c>
       <c r="B43" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C43" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/aanvraag_schrapping_niet_aanvaard</v>
       </c>
       <c r="D43" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E43" t="str">
-        <v>beslissingsstuk</v>
+        <v>SCHR_NANVRD</v>
       </c>
       <c r="F43" t="str">
-        <v>Stuk dat voortkomt uit een beslissing</v>
+        <v>Schrapping niet aanvaard</v>
       </c>
       <c r="G43" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
+        <v>null</v>
       </c>
       <c r="H43" t="str">
         <v>null</v>
@@ -2906,19 +2906,19 @@
         <v>null</v>
       </c>
       <c r="J43" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
       </c>
       <c r="K43" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
       </c>
       <c r="L43" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_niet_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_niet_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_niet_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_niet_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_ingewilligd|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_ingewilligd_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_onontvankelijk_verklaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_onontvankelijk_verklaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_verworpen|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_verworpen_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/registratieattest|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/registratieattest_begeleidende_brief</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
       </c>
       <c r="M43" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_niet_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_niet_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_niet_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_niet_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_ingewilligd|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_ingewilligd_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_onontvankelijk_verklaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_onontvankelijk_verklaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_verworpen|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_verworpen_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/registratieattest|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/registratieattest_begeleidende_brief</v>
+        <v>null</v>
       </c>
       <c r="N43" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_niet_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_niet_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_niet_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_niet_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_ingewilligd|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_ingewilligd_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_onontvankelijk_verklaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_onontvankelijk_verklaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_verworpen|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_verworpen_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/registratieattest|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/registratieattest_begeleidende_brief</v>
+        <v>null</v>
       </c>
       <c r="O43" t="str">
         <v>null</v>
@@ -2938,22 +2938,22 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/foto</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_niet_aanvaard_begeleidende_brief</v>
       </c>
       <c r="B44" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C44" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_niet_aanvaard</v>
       </c>
       <c r="D44" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E44" t="str">
-        <v>FOTO</v>
+        <v>SCHR_NANVRD_BEG_BRIEF</v>
       </c>
       <c r="F44" t="str">
-        <v>Foto</v>
+        <v>Begeleidende brief bij schrapping niet aanvaard</v>
       </c>
       <c r="G44" t="str">
         <v>null</v>
@@ -2965,13 +2965,13 @@
         <v>null</v>
       </c>
       <c r="J44" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/stavingsstuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
       </c>
       <c r="K44" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/stavingsstuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
       </c>
       <c r="L44" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/stavingsstuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
       </c>
       <c r="M44" t="str">
         <v>null</v>
@@ -2997,22 +2997,22 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/inkomend_procedurestuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_ingewilligd</v>
       </c>
       <c r="B45" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C45" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/beroep_tegen_registratie_ingewilligd</v>
       </c>
       <c r="D45" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E45" t="str">
-        <v>INKOMEND_PROCEDURESTUK</v>
+        <v>BER_INGWD</v>
       </c>
       <c r="F45" t="str">
-        <v>Inkomend procedurestuk</v>
+        <v>Beroep ingewilligd</v>
       </c>
       <c r="G45" t="str">
         <v>null</v>
@@ -3024,13 +3024,13 @@
         <v>null</v>
       </c>
       <c r="J45" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/procedurestuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
       </c>
       <c r="K45" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/procedurestuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
       </c>
       <c r="L45" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/procedurestuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
       </c>
       <c r="M45" t="str">
         <v>null</v>
@@ -3056,25 +3056,25 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/procedurestuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_ingewilligd_begeleidende_brief</v>
       </c>
       <c r="B46" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C46" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_ingewilligd</v>
       </c>
       <c r="D46" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E46" t="str">
-        <v>procedurestuk</v>
+        <v>BER_INGWD_BEG_BRIEF</v>
       </c>
       <c r="F46" t="str">
-        <v>Stuk gerelateerd aan een procedure</v>
+        <v>Begeleidende brief bij beroep ingewilligd</v>
       </c>
       <c r="G46" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
+        <v>null</v>
       </c>
       <c r="H46" t="str">
         <v>null</v>
@@ -3083,19 +3083,19 @@
         <v>null</v>
       </c>
       <c r="J46" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
       </c>
       <c r="K46" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
       </c>
       <c r="L46" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/inkomend_procedurestuk|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/retour_afzender_procedurestuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
       </c>
       <c r="M46" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/inkomend_procedurestuk|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/retour_afzender_procedurestuk</v>
+        <v>null</v>
       </c>
       <c r="N46" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/inkomend_procedurestuk|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/retour_afzender_procedurestuk</v>
+        <v>null</v>
       </c>
       <c r="O46" t="str">
         <v>null</v>
@@ -3115,22 +3115,22 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/registratieattest</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_onontvankelijk_verklaard</v>
       </c>
       <c r="B47" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C47" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/geregistreerd_in_inventaris</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/beroep_tegen_registratie_onontvankelijk_verklaard</v>
       </c>
       <c r="D47" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E47" t="str">
-        <v>REGATT</v>
+        <v>BER_ON</v>
       </c>
       <c r="F47" t="str">
-        <v>Registratieattest</v>
+        <v>Beroep onontvankelijk verklaard</v>
       </c>
       <c r="G47" t="str">
         <v>null</v>
@@ -3174,22 +3174,22 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/registratieattest_begeleidende_brief</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_onontvankelijk_verklaard_begeleidende_brief</v>
       </c>
       <c r="B48" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C48" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_onontvankelijk_verklaard</v>
       </c>
       <c r="D48" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E48" t="str">
-        <v>REGATT_BEG_BRIEF</v>
+        <v>BER_ON_BEG_BRIEF</v>
       </c>
       <c r="F48" t="str">
-        <v>Begeleidende brief bij een registratieattest</v>
+        <v>Begeleidende brief bij beroep onontvankelijk verklaard</v>
       </c>
       <c r="G48" t="str">
         <v>null</v>
@@ -3233,22 +3233,22 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/retour_afzender_procedurestuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_verworpen</v>
       </c>
       <c r="B49" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C49" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/beroep_tegen_registratie_verworpen</v>
       </c>
       <c r="D49" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E49" t="str">
-        <v>RETOUR_AFZENDER_PROCEDURESTUK</v>
+        <v>BER_VERWN</v>
       </c>
       <c r="F49" t="str">
-        <v>Retour afzender</v>
+        <v>Beroep verworpen</v>
       </c>
       <c r="G49" t="str">
         <v>null</v>
@@ -3260,13 +3260,13 @@
         <v>null</v>
       </c>
       <c r="J49" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/procedurestuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
       </c>
       <c r="K49" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/procedurestuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
       </c>
       <c r="L49" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/procedurestuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
       </c>
       <c r="M49" t="str">
         <v>null</v>
@@ -3292,25 +3292,25 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/stavingsstuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_verworpen_begeleidende_brief</v>
       </c>
       <c r="B50" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C50" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_verworpen</v>
       </c>
       <c r="D50" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E50" t="str">
-        <v>stavingsstuk</v>
+        <v>BER_VERWN_BEG_BRIEF</v>
       </c>
       <c r="F50" t="str">
-        <v>Stavingsstuk bij een vaststelling</v>
+        <v>Begeleidende brief bij beroep verworpen</v>
       </c>
       <c r="G50" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
+        <v>null</v>
       </c>
       <c r="H50" t="str">
         <v>null</v>
@@ -3319,19 +3319,19 @@
         <v>null</v>
       </c>
       <c r="J50" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
       </c>
       <c r="K50" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
       </c>
       <c r="L50" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/foto|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/varia|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/verslag</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
       </c>
       <c r="M50" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/foto|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/varia|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/verslag</v>
+        <v>null</v>
       </c>
       <c r="N50" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/foto|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/varia|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/verslag</v>
+        <v>null</v>
       </c>
       <c r="O50" t="str">
         <v>null</v>
@@ -3351,7 +3351,7 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/varia</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
       </c>
       <c r="B51" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -3363,13 +3363,13 @@
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E51" t="str">
-        <v>VARIA</v>
+        <v>beslissingsstuk</v>
       </c>
       <c r="F51" t="str">
-        <v>Varia</v>
+        <v>Stuk dat voortkomt uit een beslissing</v>
       </c>
       <c r="G51" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="H51" t="str">
         <v>null</v>
@@ -3378,19 +3378,19 @@
         <v>null</v>
       </c>
       <c r="J51" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/stavingsstuk</v>
+        <v>null</v>
       </c>
       <c r="K51" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/stavingsstuk</v>
+        <v>null</v>
       </c>
       <c r="L51" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/stavingsstuk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_niet_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_niet_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_niet_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_niet_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_ingewilligd|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_ingewilligd_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_onontvankelijk_verklaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_onontvankelijk_verklaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_verworpen|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_verworpen_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/registratieattest|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/registratieattest_begeleidende_brief</v>
       </c>
       <c r="M51" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_niet_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_niet_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_niet_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_niet_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_ingewilligd|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_ingewilligd_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_onontvankelijk_verklaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_onontvankelijk_verklaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_verworpen|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_verworpen_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/registratieattest|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/registratieattest_begeleidende_brief</v>
       </c>
       <c r="N51" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_niet_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_opschorting_heffing_niet_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_niet_aanvaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/aanvraag_schrapping_niet_aanvaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_ingewilligd|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_ingewilligd_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_onontvankelijk_verklaard|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_onontvankelijk_verklaard_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_verworpen|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beroep_tegen_registratie_verworpen_begeleidende_brief|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/registratieattest|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/registratieattest_begeleidende_brief</v>
       </c>
       <c r="O51" t="str">
         <v>null</v>
@@ -3410,7 +3410,7 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/verslag</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/foto</v>
       </c>
       <c r="B52" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -3422,10 +3422,10 @@
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E52" t="str">
-        <v>VERSLAG</v>
+        <v>FOTO</v>
       </c>
       <c r="F52" t="str">
-        <v>Verslag</v>
+        <v>Foto</v>
       </c>
       <c r="G52" t="str">
         <v>null</v>
@@ -3469,7 +3469,7 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/buitenmuren</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/inkomend_procedurestuk</v>
       </c>
       <c r="B53" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -3478,13 +3478,13 @@
         <v>null</v>
       </c>
       <c r="D53" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/uitgesproken_gebrek</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E53" t="str">
-        <v>buitenmuren</v>
+        <v>INKOMEND_PROCEDURESTUK</v>
       </c>
       <c r="F53" t="str">
-        <v>Gebrek aan de toestand van buitenmuren</v>
+        <v>Inkomend procedurestuk</v>
       </c>
       <c r="G53" t="str">
         <v>null</v>
@@ -3496,13 +3496,13 @@
         <v>null</v>
       </c>
       <c r="J53" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/procedurestuk</v>
       </c>
       <c r="K53" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/procedurestuk</v>
       </c>
       <c r="L53" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/procedurestuk</v>
       </c>
       <c r="M53" t="str">
         <v>null</v>
@@ -3511,13 +3511,13 @@
         <v>null</v>
       </c>
       <c r="O53" t="str">
-        <v>Buitenmuren</v>
+        <v>null</v>
       </c>
       <c r="P53" t="str">
-        <v>http://www.eionet.europa.eu/gemet/theme/5</v>
+        <v>null</v>
       </c>
       <c r="Q53" t="str">
-        <v>https://data.omgeving.vlaanderen.be/ns/verwaarlozing#vertoont_gebrek_ivm_buitenmuren</v>
+        <v>null</v>
       </c>
       <c r="R53" t="str">
         <v>null</v>
@@ -3528,7 +3528,7 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/buitentimmerwerk</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/procedurestuk</v>
       </c>
       <c r="B54" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -3537,16 +3537,16 @@
         <v>null</v>
       </c>
       <c r="D54" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/uitgesproken_gebrek</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E54" t="str">
-        <v>buitentimmerwerk</v>
+        <v>procedurestuk</v>
       </c>
       <c r="F54" t="str">
-        <v>Gebrek aan de toestand van het buitentimmerwerk</v>
+        <v>Stuk gerelateerd aan een procedure</v>
       </c>
       <c r="G54" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="H54" t="str">
         <v>null</v>
@@ -3555,28 +3555,28 @@
         <v>null</v>
       </c>
       <c r="J54" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
+        <v>null</v>
       </c>
       <c r="K54" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
+        <v>null</v>
       </c>
       <c r="L54" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/inkomend_procedurestuk|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/retour_afzender_procedurestuk</v>
       </c>
       <c r="M54" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/inkomend_procedurestuk|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/retour_afzender_procedurestuk</v>
       </c>
       <c r="N54" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/inkomend_procedurestuk|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/retour_afzender_procedurestuk</v>
       </c>
       <c r="O54" t="str">
-        <v>Buitentimmerwerk</v>
+        <v>null</v>
       </c>
       <c r="P54" t="str">
-        <v>http://www.eionet.europa.eu/gemet/theme/5</v>
+        <v>null</v>
       </c>
       <c r="Q54" t="str">
-        <v>https://data.omgeving.vlaanderen.be/ns/verwaarlozing#vertoont_gebrek_ivm_buitentimmerwerk</v>
+        <v>null</v>
       </c>
       <c r="R54" t="str">
         <v>null</v>
@@ -3587,22 +3587,22 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakbedekking</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/registratieattest</v>
       </c>
       <c r="B55" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C55" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/beslissing/geregistreerd_in_inventaris</v>
       </c>
       <c r="D55" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/uitgesproken_gebrek</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E55" t="str">
-        <v>dakbedekking</v>
+        <v>REGATT</v>
       </c>
       <c r="F55" t="str">
-        <v>Gebrek aan de toestand van de dakbedekking</v>
+        <v>Registratieattest</v>
       </c>
       <c r="G55" t="str">
         <v>null</v>
@@ -3614,13 +3614,13 @@
         <v>null</v>
       </c>
       <c r="J55" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
       </c>
       <c r="K55" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
       </c>
       <c r="L55" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
       </c>
       <c r="M55" t="str">
         <v>null</v>
@@ -3629,13 +3629,13 @@
         <v>null</v>
       </c>
       <c r="O55" t="str">
-        <v>Dakbedekking</v>
+        <v>null</v>
       </c>
       <c r="P55" t="str">
-        <v>http://www.eionet.europa.eu/gemet/theme/5</v>
+        <v>null</v>
       </c>
       <c r="Q55" t="str">
-        <v>https://data.omgeving.vlaanderen.be/ns/verwaarlozing#vertoont_gebrek_ivm_dakbedekking</v>
+        <v>null</v>
       </c>
       <c r="R55" t="str">
         <v>null</v>
@@ -3646,7 +3646,7 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakgebinte</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/registratieattest_begeleidende_brief</v>
       </c>
       <c r="B56" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -3655,13 +3655,13 @@
         <v>null</v>
       </c>
       <c r="D56" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/uitgesproken_gebrek</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E56" t="str">
-        <v>dakgebinte</v>
+        <v>REGATT_BEG_BRIEF</v>
       </c>
       <c r="F56" t="str">
-        <v>Gebrek aan de toestand van het dakgebinte</v>
+        <v>Begeleidende brief bij een registratieattest</v>
       </c>
       <c r="G56" t="str">
         <v>null</v>
@@ -3673,13 +3673,13 @@
         <v>null</v>
       </c>
       <c r="J56" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
       </c>
       <c r="K56" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
       </c>
       <c r="L56" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/beslissingsstuk</v>
       </c>
       <c r="M56" t="str">
         <v>null</v>
@@ -3688,13 +3688,13 @@
         <v>null</v>
       </c>
       <c r="O56" t="str">
-        <v>Dakgebinte</v>
+        <v>null</v>
       </c>
       <c r="P56" t="str">
-        <v>http://www.eionet.europa.eu/gemet/theme/5</v>
+        <v>null</v>
       </c>
       <c r="Q56" t="str">
-        <v>https://data.omgeving.vlaanderen.be/ns/verwaarlozing#vertoont_gebrek_ivm_dakgebinte</v>
+        <v>null</v>
       </c>
       <c r="R56" t="str">
         <v>null</v>
@@ -3705,7 +3705,7 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakgoten</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/retour_afzender_procedurestuk</v>
       </c>
       <c r="B57" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -3714,13 +3714,13 @@
         <v>null</v>
       </c>
       <c r="D57" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/uitgesproken_gebrek</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E57" t="str">
-        <v>dakgoten</v>
+        <v>RETOUR_AFZENDER_PROCEDURESTUK</v>
       </c>
       <c r="F57" t="str">
-        <v>Gebrek aan de toestand van de dakgoten</v>
+        <v>Retour afzender</v>
       </c>
       <c r="G57" t="str">
         <v>null</v>
@@ -3732,13 +3732,13 @@
         <v>null</v>
       </c>
       <c r="J57" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/procedurestuk</v>
       </c>
       <c r="K57" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/procedurestuk</v>
       </c>
       <c r="L57" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/procedurestuk</v>
       </c>
       <c r="M57" t="str">
         <v>null</v>
@@ -3747,13 +3747,13 @@
         <v>null</v>
       </c>
       <c r="O57" t="str">
-        <v>Dakgoten</v>
+        <v>null</v>
       </c>
       <c r="P57" t="str">
-        <v>http://www.eionet.europa.eu/gemet/theme/5</v>
+        <v>null</v>
       </c>
       <c r="Q57" t="str">
-        <v>https://data.omgeving.vlaanderen.be/ns/verwaarlozing#vertoont_gebrek_ivm_dakgoten</v>
+        <v>null</v>
       </c>
       <c r="R57" t="str">
         <v>null</v>
@@ -3764,7 +3764,7 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/stavingsstuk</v>
       </c>
       <c r="B58" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -3773,16 +3773,16 @@
         <v>null</v>
       </c>
       <c r="D58" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/uitgesproken_gebrek</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E58" t="str">
-        <v>gebouwonderdeel</v>
+        <v>stavingsstuk</v>
       </c>
       <c r="F58" t="str">
-        <v>Gebrek aan de toestand van een gebouwonderdeel</v>
+        <v>Stavingsstuk bij een vaststelling</v>
       </c>
       <c r="G58" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/uitgesproken_gebrek</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="H58" t="str">
         <v>null</v>
@@ -3797,22 +3797,22 @@
         <v>null</v>
       </c>
       <c r="L58" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/buitenmuren|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/buitentimmerwerk|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakbedekking|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakgebinte|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakgoten|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/kroonlijst|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/liften|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/schoorstenen|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/trappen</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/foto|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/varia|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/verslag</v>
       </c>
       <c r="M58" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/buitenmuren|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/buitentimmerwerk|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakbedekking|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakgebinte|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakgoten|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/kroonlijst|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/liften|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/schoorstenen|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/trappen</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/foto|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/varia|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/verslag</v>
       </c>
       <c r="N58" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/buitenmuren|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/buitentimmerwerk|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakbedekking|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakgebinte|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakgoten|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/kroonlijst|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/liften|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/schoorstenen|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/trappen</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/foto|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/varia|https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/verslag</v>
       </c>
       <c r="O58" t="str">
-        <v>Gebrek aan de toestand van een gebouwonderdeel</v>
+        <v>null</v>
       </c>
       <c r="P58" t="str">
-        <v>http://www.eionet.europa.eu/gemet/theme/5</v>
+        <v>null</v>
       </c>
       <c r="Q58" t="str">
-        <v>https://data.omgeving.vlaanderen.be/ns/verwaarlozing#vertoont_gebrek_ivm_gebouwonderdeel</v>
+        <v>null</v>
       </c>
       <c r="R58" t="str">
         <v>null</v>
@@ -3823,7 +3823,7 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/kroonlijst</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/varia</v>
       </c>
       <c r="B59" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -3832,13 +3832,13 @@
         <v>null</v>
       </c>
       <c r="D59" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/uitgesproken_gebrek</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E59" t="str">
-        <v>kroonlijst</v>
+        <v>VARIA</v>
       </c>
       <c r="F59" t="str">
-        <v>Gebrek aan de toestand van de kroonlijst</v>
+        <v>Varia</v>
       </c>
       <c r="G59" t="str">
         <v>null</v>
@@ -3850,13 +3850,13 @@
         <v>null</v>
       </c>
       <c r="J59" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/stavingsstuk</v>
       </c>
       <c r="K59" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/stavingsstuk</v>
       </c>
       <c r="L59" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/stavingsstuk</v>
       </c>
       <c r="M59" t="str">
         <v>null</v>
@@ -3865,13 +3865,13 @@
         <v>null</v>
       </c>
       <c r="O59" t="str">
-        <v>Kroonlijst</v>
+        <v>null</v>
       </c>
       <c r="P59" t="str">
-        <v>http://www.eionet.europa.eu/gemet/theme/5</v>
+        <v>null</v>
       </c>
       <c r="Q59" t="str">
-        <v>https://data.omgeving.vlaanderen.be/ns/verwaarlozing#vertoont_gebrek_ivm_kroonlijst</v>
+        <v>null</v>
       </c>
       <c r="R59" t="str">
         <v>null</v>
@@ -3882,7 +3882,7 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/liften</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/verslag</v>
       </c>
       <c r="B60" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -3891,13 +3891,13 @@
         <v>null</v>
       </c>
       <c r="D60" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/uitgesproken_gebrek</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/stuk</v>
       </c>
       <c r="E60" t="str">
-        <v>liften</v>
+        <v>VERSLAG</v>
       </c>
       <c r="F60" t="str">
-        <v>Gebrek aan de toestand van de liften</v>
+        <v>Verslag</v>
       </c>
       <c r="G60" t="str">
         <v>null</v>
@@ -3909,13 +3909,13 @@
         <v>null</v>
       </c>
       <c r="J60" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/stavingsstuk</v>
       </c>
       <c r="K60" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/stavingsstuk</v>
       </c>
       <c r="L60" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/stuk/stavingsstuk</v>
       </c>
       <c r="M60" t="str">
         <v>null</v>
@@ -3924,13 +3924,13 @@
         <v>null</v>
       </c>
       <c r="O60" t="str">
-        <v>Liften</v>
+        <v>null</v>
       </c>
       <c r="P60" t="str">
-        <v>http://www.eionet.europa.eu/gemet/theme/5</v>
+        <v>null</v>
       </c>
       <c r="Q60" t="str">
-        <v>https://data.omgeving.vlaanderen.be/ns/verwaarlozing#vertoont_gebrek_ivm_liften</v>
+        <v>null</v>
       </c>
       <c r="R60" t="str">
         <v>null</v>
@@ -3941,7 +3941,7 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/reden_van_verwijderen_uit_inventaris:benutting_meer_dan_vijftig_percent</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/buitenmuren</v>
       </c>
       <c r="B61" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -3950,16 +3950,16 @@
         <v>null</v>
       </c>
       <c r="D61" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/reden_van_verwijderen_uit_inventaris</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/uitgesproken_gebrek</v>
       </c>
       <c r="E61" t="str">
-        <v>+50%</v>
+        <v>buitenmuren</v>
       </c>
       <c r="F61" t="str">
-        <v>Benutting van meer dan 50% conform de vergunde bestemming van het gebouw</v>
+        <v>Gebrek aan de toestand van buitenmuren</v>
       </c>
       <c r="G61" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/reden_van_verwijderen_uit_inventaris</v>
+        <v>null</v>
       </c>
       <c r="H61" t="str">
         <v>null</v>
@@ -3968,13 +3968,13 @@
         <v>null</v>
       </c>
       <c r="J61" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
       </c>
       <c r="K61" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
       </c>
       <c r="L61" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
       </c>
       <c r="M61" t="str">
         <v>null</v>
@@ -3983,13 +3983,13 @@
         <v>null</v>
       </c>
       <c r="O61" t="str">
-        <v>null</v>
+        <v>Buitenmuren</v>
       </c>
       <c r="P61" t="str">
-        <v>null</v>
+        <v>http://www.eionet.europa.eu/gemet/theme/5</v>
       </c>
       <c r="Q61" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/ns/verwaarlozing#vertoont_gebrek_ivm_buitenmuren</v>
       </c>
       <c r="R61" t="str">
         <v>null</v>
@@ -4000,7 +4000,7 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/reden_van_verwijderen_uit_inventaris:functiewijziging</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/buitentimmerwerk</v>
       </c>
       <c r="B62" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -4009,16 +4009,16 @@
         <v>null</v>
       </c>
       <c r="D62" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/reden_van_verwijderen_uit_inventaris</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/uitgesproken_gebrek</v>
       </c>
       <c r="E62" t="str">
-        <v>functiewijziging</v>
+        <v>buitentimmerwerk</v>
       </c>
       <c r="F62" t="str">
-        <v>Functiewijziging doorgevoerd</v>
+        <v>Gebrek aan de toestand van het buitentimmerwerk</v>
       </c>
       <c r="G62" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/reden_van_verwijderen_uit_inventaris</v>
+        <v>null</v>
       </c>
       <c r="H62" t="str">
         <v>null</v>
@@ -4027,13 +4027,13 @@
         <v>null</v>
       </c>
       <c r="J62" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
       </c>
       <c r="K62" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
       </c>
       <c r="L62" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
       </c>
       <c r="M62" t="str">
         <v>null</v>
@@ -4042,13 +4042,13 @@
         <v>null</v>
       </c>
       <c r="O62" t="str">
-        <v>null</v>
+        <v>Buitentimmerwerk</v>
       </c>
       <c r="P62" t="str">
-        <v>null</v>
+        <v>http://www.eionet.europa.eu/gemet/theme/5</v>
       </c>
       <c r="Q62" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/ns/verwaarlozing#vertoont_gebrek_ivm_buitentimmerwerk</v>
       </c>
       <c r="R62" t="str">
         <v>null</v>
@@ -4059,7 +4059,7 @@
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/reden_van_verwijderen_uit_inventaris:gesloopt</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakbedekking</v>
       </c>
       <c r="B63" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -4068,16 +4068,16 @@
         <v>null</v>
       </c>
       <c r="D63" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/reden_van_verwijderen_uit_inventaris</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/uitgesproken_gebrek</v>
       </c>
       <c r="E63" t="str">
-        <v>gesloopt</v>
+        <v>dakbedekking</v>
       </c>
       <c r="F63" t="str">
-        <v>De bedrijfsruimte is gesloopt</v>
+        <v>Gebrek aan de toestand van de dakbedekking</v>
       </c>
       <c r="G63" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/reden_van_verwijderen_uit_inventaris</v>
+        <v>null</v>
       </c>
       <c r="H63" t="str">
         <v>null</v>
@@ -4086,13 +4086,13 @@
         <v>null</v>
       </c>
       <c r="J63" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
       </c>
       <c r="K63" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
       </c>
       <c r="L63" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
       </c>
       <c r="M63" t="str">
         <v>null</v>
@@ -4101,13 +4101,13 @@
         <v>null</v>
       </c>
       <c r="O63" t="str">
-        <v>null</v>
+        <v>Dakbedekking</v>
       </c>
       <c r="P63" t="str">
-        <v>null</v>
+        <v>http://www.eionet.europa.eu/gemet/theme/5</v>
       </c>
       <c r="Q63" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/ns/verwaarlozing#vertoont_gebrek_ivm_dakbedekking</v>
       </c>
       <c r="R63" t="str">
         <v>null</v>
@@ -4118,7 +4118,7 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/reden_van_verwijderen_uit_inventaris:heffing</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakgebinte</v>
       </c>
       <c r="B64" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -4127,16 +4127,16 @@
         <v>null</v>
       </c>
       <c r="D64" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/reden_van_verwijderen_uit_inventaris</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/uitgesproken_gebrek</v>
       </c>
       <c r="E64" t="str">
-        <v>heffing</v>
+        <v>dakgebinte</v>
       </c>
       <c r="F64" t="str">
-        <v>Procedure heffing</v>
+        <v>Gebrek aan de toestand van het dakgebinte</v>
       </c>
       <c r="G64" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/reden_van_verwijderen_uit_inventaris</v>
+        <v>null</v>
       </c>
       <c r="H64" t="str">
         <v>null</v>
@@ -4145,13 +4145,13 @@
         <v>null</v>
       </c>
       <c r="J64" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
       </c>
       <c r="K64" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
       </c>
       <c r="L64" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
       </c>
       <c r="M64" t="str">
         <v>null</v>
@@ -4160,13 +4160,13 @@
         <v>null</v>
       </c>
       <c r="O64" t="str">
-        <v>null</v>
+        <v>Dakgebinte</v>
       </c>
       <c r="P64" t="str">
-        <v>null</v>
+        <v>http://www.eionet.europa.eu/gemet/theme/5</v>
       </c>
       <c r="Q64" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/ns/verwaarlozing#vertoont_gebrek_ivm_dakgebinte</v>
       </c>
       <c r="R64" t="str">
         <v>null</v>
@@ -4177,7 +4177,7 @@
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/reden_van_verwijderen_uit_inventaris:nieuwe_invulling</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakgoten</v>
       </c>
       <c r="B65" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -4186,16 +4186,16 @@
         <v>null</v>
       </c>
       <c r="D65" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/reden_van_verwijderen_uit_inventaris</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/uitgesproken_gebrek</v>
       </c>
       <c r="E65" t="str">
-        <v>nieuwe_invulling</v>
+        <v>dakgoten</v>
       </c>
       <c r="F65" t="str">
-        <v>Nieuwe invulling gegeven conform de vergunde bestemming</v>
+        <v>Gebrek aan de toestand van de dakgoten</v>
       </c>
       <c r="G65" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/reden_van_verwijderen_uit_inventaris</v>
+        <v>null</v>
       </c>
       <c r="H65" t="str">
         <v>null</v>
@@ -4204,13 +4204,13 @@
         <v>null</v>
       </c>
       <c r="J65" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
       </c>
       <c r="K65" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
       </c>
       <c r="L65" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
       </c>
       <c r="M65" t="str">
         <v>null</v>
@@ -4219,13 +4219,13 @@
         <v>null</v>
       </c>
       <c r="O65" t="str">
-        <v>null</v>
+        <v>Dakgoten</v>
       </c>
       <c r="P65" t="str">
-        <v>null</v>
+        <v>http://www.eionet.europa.eu/gemet/theme/5</v>
       </c>
       <c r="Q65" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/ns/verwaarlozing#vertoont_gebrek_ivm_dakgoten</v>
       </c>
       <c r="R65" t="str">
         <v>null</v>
@@ -4236,7 +4236,7 @@
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/reden_van_verwijderen_uit_inventaris:onteigening</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
       </c>
       <c r="B66" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -4245,16 +4245,16 @@
         <v>null</v>
       </c>
       <c r="D66" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/reden_van_verwijderen_uit_inventaris</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/uitgesproken_gebrek</v>
       </c>
       <c r="E66" t="str">
-        <v>onteigening</v>
+        <v>gebouwonderdeel</v>
       </c>
       <c r="F66" t="str">
-        <v>Er is een onteigening</v>
+        <v>Gebrek aan de toestand van een gebouwonderdeel</v>
       </c>
       <c r="G66" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/reden_van_verwijderen_uit_inventaris</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/uitgesproken_gebrek</v>
       </c>
       <c r="H66" t="str">
         <v>null</v>
@@ -4269,22 +4269,22 @@
         <v>null</v>
       </c>
       <c r="L66" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/buitenmuren|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/buitentimmerwerk|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakbedekking|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakgebinte|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakgoten|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/kroonlijst|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/liften|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/schoorstenen|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/trappen</v>
       </c>
       <c r="M66" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/buitenmuren|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/buitentimmerwerk|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakbedekking|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakgebinte|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakgoten|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/kroonlijst|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/liften|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/schoorstenen|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/trappen</v>
       </c>
       <c r="N66" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/buitenmuren|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/buitentimmerwerk|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakbedekking|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakgebinte|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/dakgoten|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/kroonlijst|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/liften|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/schoorstenen|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/trappen</v>
       </c>
       <c r="O66" t="str">
-        <v>null</v>
+        <v>Gebrek aan de toestand van een gebouwonderdeel</v>
       </c>
       <c r="P66" t="str">
-        <v>null</v>
+        <v>http://www.eionet.europa.eu/gemet/theme/5</v>
       </c>
       <c r="Q66" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/ns/verwaarlozing#vertoont_gebrek_ivm_gebouwonderdeel</v>
       </c>
       <c r="R66" t="str">
         <v>null</v>
@@ -4295,7 +4295,7 @@
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/reden_van_verwijderen_uit_inventaris:opgeheven</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/kroonlijst</v>
       </c>
       <c r="B67" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -4304,16 +4304,16 @@
         <v>null</v>
       </c>
       <c r="D67" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/reden_van_verwijderen_uit_inventaris</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/uitgesproken_gebrek</v>
       </c>
       <c r="E67" t="str">
-        <v>opgeheven</v>
+        <v>kroonlijst</v>
       </c>
       <c r="F67" t="str">
-        <v>Verwaarlozing is opgeheven</v>
+        <v>Gebrek aan de toestand van de kroonlijst</v>
       </c>
       <c r="G67" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/reden_van_verwijderen_uit_inventaris</v>
+        <v>null</v>
       </c>
       <c r="H67" t="str">
         <v>null</v>
@@ -4322,13 +4322,13 @@
         <v>null</v>
       </c>
       <c r="J67" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
       </c>
       <c r="K67" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
       </c>
       <c r="L67" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
       </c>
       <c r="M67" t="str">
         <v>null</v>
@@ -4337,13 +4337,13 @@
         <v>null</v>
       </c>
       <c r="O67" t="str">
-        <v>null</v>
+        <v>Kroonlijst</v>
       </c>
       <c r="P67" t="str">
-        <v>null</v>
+        <v>http://www.eionet.europa.eu/gemet/theme/5</v>
       </c>
       <c r="Q67" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/ns/verwaarlozing#vertoont_gebrek_ivm_kroonlijst</v>
       </c>
       <c r="R67" t="str">
         <v>null</v>
@@ -4354,7 +4354,7 @@
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/reden_van_verwijderen_uit_inventaris:rechtbank</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/liften</v>
       </c>
       <c r="B68" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -4363,16 +4363,16 @@
         <v>null</v>
       </c>
       <c r="D68" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/reden_van_verwijderen_uit_inventaris</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/uitgesproken_gebrek</v>
       </c>
       <c r="E68" t="str">
-        <v>rechtbank</v>
+        <v>liften</v>
       </c>
       <c r="F68" t="str">
-        <v>Procedure rechtbank</v>
+        <v>Gebrek aan de toestand van de liften</v>
       </c>
       <c r="G68" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/leegstand/reden_van_verwijderen_uit_inventaris</v>
+        <v>null</v>
       </c>
       <c r="H68" t="str">
         <v>null</v>
@@ -4381,13 +4381,13 @@
         <v>null</v>
       </c>
       <c r="J68" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
       </c>
       <c r="K68" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
       </c>
       <c r="L68" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/gebouwonderdeel</v>
       </c>
       <c r="M68" t="str">
         <v>null</v>
@@ -4396,13 +4396,13 @@
         <v>null</v>
       </c>
       <c r="O68" t="str">
-        <v>null</v>
+        <v>Liften</v>
       </c>
       <c r="P68" t="str">
-        <v>null</v>
+        <v>http://www.eionet.europa.eu/gemet/theme/5</v>
       </c>
       <c r="Q68" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/ns/verwaarlozing#vertoont_gebrek_ivm_liften</v>
       </c>
       <c r="R68" t="str">
         <v>null</v>
@@ -4939,7 +4939,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/dataset/codelijst-verwaarlozing</v>
       </c>
       <c r="S77" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/reden_van_verwijderen_uit_inventaris:benutting_meer_dan_vijftig_percent|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/reden_van_verwijderen_uit_inventaris:functiewijziging|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/reden_van_verwijderen_uit_inventaris:gesloopt|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/reden_van_verwijderen_uit_inventaris:heffing|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/reden_van_verwijderen_uit_inventaris:nieuwe_invulling|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/reden_van_verwijderen_uit_inventaris:onteigening|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/reden_van_verwijderen_uit_inventaris:opgeheven|https://data.omgeving.vlaanderen.be/id/concept/leegstand/uitgesproken_gebrek/reden_van_verwijderen_uit_inventaris:rechtbank</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/leegstand/reden_van_verwijderen_uit_inventaris/benutting_meer_dan_vijftig_percent|https://data.omgeving.vlaanderen.be/id/concept/leegstand/reden_van_verwijderen_uit_inventaris/functiewijziging|https://data.omgeving.vlaanderen.be/id/concept/leegstand/reden_van_verwijderen_uit_inventaris/gesloopt|https://data.omgeving.vlaanderen.be/id/concept/leegstand/reden_van_verwijderen_uit_inventaris/heffing|https://data.omgeving.vlaanderen.be/id/concept/leegstand/reden_van_verwijderen_uit_inventaris/nieuwe_invulling|https://data.omgeving.vlaanderen.be/id/concept/leegstand/reden_van_verwijderen_uit_inventaris/onteigening|https://data.omgeving.vlaanderen.be/id/concept/leegstand/reden_van_verwijderen_uit_inventaris/opgeheven|https://data.omgeving.vlaanderen.be/id/concept/leegstand/reden_van_verwijderen_uit_inventaris/rechtbank</v>
       </c>
     </row>
     <row r="78">

</xml_diff>